<commit_message>
Add Sweco Munich (BIM Coordinator TGA) row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2495,28 +2495,66 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="21">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="11" t="n"/>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
-      <c r="H22" s="13" t="n"/>
-      <c r="I22" s="12" t="n"/>
-      <c r="J22" s="12" t="n"/>
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>BIM Coordinator – Technical Building Equipment (m/f/x), Job No. S2921</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Munich, DE</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr"/>
+      <c r="E22" s="17" t="inlineStr"/>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco-services.de/bms.nsf/Bewerbung?openform&amp;job=S2921</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="n">
+        <v>46237</v>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr"/>
       <c r="K22" s="14">
         <f>IF($H22="","",TODAY()-$H22)</f>
         <v/>
       </c>
-      <c r="L22" s="13" t="n"/>
-      <c r="M22" s="11" t="n"/>
-      <c r="N22" s="13" t="n"/>
-      <c r="O22" s="11" t="n"/>
-      <c r="P22" s="11" t="n"/>
-      <c r="Q22" s="11" t="n"/>
-      <c r="R22" s="12" t="n"/>
-      <c r="S22" s="11" t="n"/>
+      <c r="L22" s="19" t="inlineStr"/>
+      <c r="M22" s="17" t="inlineStr"/>
+      <c r="N22" s="19" t="inlineStr"/>
+      <c r="O22" s="17" t="inlineStr"/>
+      <c r="P22" s="17" t="inlineStr"/>
+      <c r="Q22" s="17" t="inlineStr">
+        <is>
+          <t>germany/2026_08_03_sweco_munich_bim_coordinator</t>
+        </is>
+      </c>
+      <c r="R22" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S22" s="17" t="inlineStr">
+        <is>
+          <t>Stacked gaps: several years experience required, LINEAR/ALPI software not held, German mandatory (candidate has none). Applied anyway, honest about all three. First German-market CV variant (DOB/nationality added, MM.YYYY dates, no photo — flagged not fabricated).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="21">
       <c r="A23" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Bayards Aluminium Solutions row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2557,28 +2557,66 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="21">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
-      <c r="H23" s="13" t="n"/>
-      <c r="I23" s="12" t="n"/>
-      <c r="J23" s="12" t="n"/>
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Bayards Aluminium Solutions</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Cost Proposal Engineer – Aluminium Solutions</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Nieuw-Lekkerland, NL</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr"/>
+      <c r="E23" s="17" t="inlineStr"/>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr"/>
+      <c r="H23" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I23" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J23" s="18" t="inlineStr"/>
       <c r="K23" s="14">
         <f>IF($H23="","",TODAY()-$H23)</f>
         <v/>
       </c>
-      <c r="L23" s="13" t="n"/>
-      <c r="M23" s="11" t="n"/>
-      <c r="N23" s="13" t="n"/>
-      <c r="O23" s="11" t="n"/>
-      <c r="P23" s="11" t="n"/>
-      <c r="Q23" s="11" t="n"/>
-      <c r="R23" s="12" t="n"/>
-      <c r="S23" s="11" t="n"/>
+      <c r="L23" s="19" t="inlineStr"/>
+      <c r="M23" s="17" t="inlineStr"/>
+      <c r="N23" s="19" t="inlineStr"/>
+      <c r="O23" s="17" t="inlineStr"/>
+      <c r="P23" s="17" t="inlineStr">
+        <is>
+          <t>work@bayards.com</t>
+        </is>
+      </c>
+      <c r="Q23" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_bayards</t>
+        </is>
+      </c>
+      <c r="R23" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S23" s="17" t="inlineStr">
+        <is>
+          <t>Strong content match (5D QTO coursework, Contract Management internship pricing/contract review). Honest that candidate has zero Dutch vs. required proficiency in both Dutch and English.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="21">
       <c r="A24" s="11" t="n"/>

</xml_diff>

<commit_message>
Mark Bayards Aluminium Solutions application as Rejected
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2588,7 +2588,11 @@
           <t>Applied</t>
         </is>
       </c>
-      <c r="J23" s="18" t="inlineStr"/>
+      <c r="J23" s="18" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="K23" s="14">
         <f>IF($H23="","",TODAY()-$H23)</f>
         <v/>

</xml_diff>

<commit_message>
Add Arup Junior Bridge Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2623,28 +2623,66 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="21">
-      <c r="A24" s="11" t="n"/>
-      <c r="B24" s="11" t="n"/>
-      <c r="C24" s="11" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="11" t="n"/>
-      <c r="F24" s="11" t="n"/>
-      <c r="G24" s="11" t="n"/>
-      <c r="H24" s="13" t="n"/>
-      <c r="I24" s="12" t="n"/>
-      <c r="J24" s="12" t="n"/>
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Arup</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Junior Bridge Engineer (Bridge &amp; Civil Structures), Job AMS000074</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Amsterdam, NL</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr"/>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr"/>
+      <c r="H24" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr"/>
       <c r="K24" s="14">
         <f>IF($H24="","",TODAY()-$H24)</f>
         <v/>
       </c>
-      <c r="L24" s="13" t="n"/>
-      <c r="M24" s="11" t="n"/>
-      <c r="N24" s="13" t="n"/>
-      <c r="O24" s="11" t="n"/>
-      <c r="P24" s="11" t="n"/>
-      <c r="Q24" s="11" t="n"/>
-      <c r="R24" s="12" t="n"/>
-      <c r="S24" s="11" t="n"/>
+      <c r="L24" s="19" t="inlineStr"/>
+      <c r="M24" s="17" t="inlineStr"/>
+      <c r="N24" s="19" t="inlineStr"/>
+      <c r="O24" s="17" t="inlineStr"/>
+      <c r="P24" s="17" t="inlineStr"/>
+      <c r="Q24" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_arup_junior_bridge_engineer</t>
+        </is>
+      </c>
+      <c r="R24" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S24" s="17" t="inlineStr">
+        <is>
+          <t>Junior-friendly seniority fit, but real gaps in FEM/structural calculations (candidate specializes in BIM coordination, not structural analysis) and Dutch B1 (candidate has none). Per user instruction, CV/letter do NOT disclose these gaps — lean only on genuine parametric-design/automation strengths.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="21">
       <c r="A25" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Arup Frankfurt Junior PM row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2685,28 +2685,66 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="21">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
-      <c r="H25" s="13" t="n"/>
-      <c r="I25" s="12" t="n"/>
-      <c r="J25" s="12" t="n"/>
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Arup</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Junior Project Manager – Science, Industry &amp; Technology</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>Frankfurt, DE</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr"/>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr"/>
+      <c r="H25" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J25" s="18" t="inlineStr"/>
       <c r="K25" s="14">
         <f>IF($H25="","",TODAY()-$H25)</f>
         <v/>
       </c>
-      <c r="L25" s="13" t="n"/>
-      <c r="M25" s="11" t="n"/>
-      <c r="N25" s="13" t="n"/>
-      <c r="O25" s="11" t="n"/>
-      <c r="P25" s="11" t="n"/>
-      <c r="Q25" s="11" t="n"/>
-      <c r="R25" s="12" t="n"/>
-      <c r="S25" s="11" t="n"/>
+      <c r="L25" s="19" t="inlineStr"/>
+      <c r="M25" s="17" t="inlineStr"/>
+      <c r="N25" s="19" t="inlineStr"/>
+      <c r="O25" s="17" t="inlineStr"/>
+      <c r="P25" s="17" t="inlineStr"/>
+      <c r="Q25" s="17" t="inlineStr">
+        <is>
+          <t>germany/2026_08_04_arup_frankfurt_junior_pm</t>
+        </is>
+      </c>
+      <c r="R25" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S25" s="17" t="inlineStr">
+        <is>
+          <t>Junior-friendly (internships/student activities explicitly welcomed). Real gap: "very good German" required, candidate has none. Per updated default, CV/letter do not disclose this gap.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="21">
       <c r="A26" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Arup Milan Assistant Computational Designer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2747,28 +2747,62 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="21">
-      <c r="A26" s="11" t="n"/>
-      <c r="B26" s="11" t="n"/>
-      <c r="C26" s="11" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="11" t="n"/>
-      <c r="F26" s="11" t="n"/>
-      <c r="G26" s="11" t="n"/>
-      <c r="H26" s="13" t="n"/>
-      <c r="I26" s="12" t="n"/>
-      <c r="J26" s="12" t="n"/>
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Arup</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Assistant Computational Designer – Digital Team</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>Milan, IT</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr"/>
+      <c r="E26" s="17" t="inlineStr"/>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr"/>
+      <c r="H26" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I26" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J26" s="18" t="inlineStr"/>
       <c r="K26" s="14">
         <f>IF($H26="","",TODAY()-$H26)</f>
         <v/>
       </c>
-      <c r="L26" s="13" t="n"/>
-      <c r="M26" s="11" t="n"/>
-      <c r="N26" s="13" t="n"/>
-      <c r="O26" s="11" t="n"/>
-      <c r="P26" s="11" t="n"/>
-      <c r="Q26" s="11" t="n"/>
-      <c r="R26" s="12" t="n"/>
-      <c r="S26" s="11" t="n"/>
+      <c r="L26" s="19" t="inlineStr"/>
+      <c r="M26" s="17" t="inlineStr"/>
+      <c r="N26" s="19" t="inlineStr"/>
+      <c r="O26" s="17" t="inlineStr"/>
+      <c r="P26" s="17" t="inlineStr"/>
+      <c r="Q26" s="17" t="inlineStr">
+        <is>
+          <t>italy/2026_08_04_arup_milan_computational_designer</t>
+        </is>
+      </c>
+      <c r="R26" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S26" s="17" t="inlineStr">
+        <is>
+          <t>Excellent fit — explicitly welcomes recent graduates, no language gap beyond English, strong overlap on Python/Dynamo/Revit/Git/AI-agent work and GIS (ArcGIS). No major mismatch to flag.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="21">
       <c r="A27" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Arup Amsterdam Design Manager row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2805,28 +2805,66 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="21">
-      <c r="A27" s="11" t="n"/>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="11" t="n"/>
-      <c r="G27" s="11" t="n"/>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="12" t="n"/>
-      <c r="J27" s="12" t="n"/>
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Arup</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Open Application – Design Manager, Private &amp; Government Property, Job AMS000091</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>Amsterdam, NL</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr"/>
+      <c r="E27" s="17" t="inlineStr"/>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>https://jobs.arup.com/jobs/33871/other-jobs-matching/location-only</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I27" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J27" s="18" t="inlineStr"/>
       <c r="K27" s="14">
         <f>IF($H27="","",TODAY()-$H27)</f>
         <v/>
       </c>
-      <c r="L27" s="13" t="n"/>
-      <c r="M27" s="11" t="n"/>
-      <c r="N27" s="13" t="n"/>
-      <c r="O27" s="11" t="n"/>
-      <c r="P27" s="11" t="n"/>
-      <c r="Q27" s="11" t="n"/>
-      <c r="R27" s="12" t="n"/>
-      <c r="S27" s="11" t="n"/>
+      <c r="L27" s="19" t="inlineStr"/>
+      <c r="M27" s="17" t="inlineStr"/>
+      <c r="N27" s="19" t="inlineStr"/>
+      <c r="O27" s="17" t="inlineStr"/>
+      <c r="P27" s="17" t="inlineStr"/>
+      <c r="Q27" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_arup_amsterdam_design_manager</t>
+        </is>
+      </c>
+      <c r="R27" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S27" s="17" t="inlineStr">
+        <is>
+          <t>Open solicitation (not a live vacancy), junior-friendly. Real gap: fluent Dutch required, candidate has none. Per updated default, CV/letter do not disclose this gap.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="21">
       <c r="A28" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Arup Amsterdam Science & Industry PM row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2867,28 +2867,66 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="21">
-      <c r="A28" s="11" t="n"/>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="11" t="n"/>
-      <c r="F28" s="11" t="n"/>
-      <c r="G28" s="11" t="n"/>
-      <c r="H28" s="13" t="n"/>
-      <c r="I28" s="12" t="n"/>
-      <c r="J28" s="12" t="n"/>
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Arup</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Open Application – Project Management, Science &amp; Industry, Job AMS000094</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>Amsterdam, NL</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr"/>
+      <c r="E28" s="17" t="inlineStr"/>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>https://jobs.arup.com/jobs/33686/other-jobs-matching/location-only</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I28" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J28" s="18" t="inlineStr"/>
       <c r="K28" s="14">
         <f>IF($H28="","",TODAY()-$H28)</f>
         <v/>
       </c>
-      <c r="L28" s="13" t="n"/>
-      <c r="M28" s="11" t="n"/>
-      <c r="N28" s="13" t="n"/>
-      <c r="O28" s="11" t="n"/>
-      <c r="P28" s="11" t="n"/>
-      <c r="Q28" s="11" t="n"/>
-      <c r="R28" s="12" t="n"/>
-      <c r="S28" s="11" t="n"/>
+      <c r="L28" s="19" t="inlineStr"/>
+      <c r="M28" s="17" t="inlineStr"/>
+      <c r="N28" s="19" t="inlineStr"/>
+      <c r="O28" s="17" t="inlineStr"/>
+      <c r="P28" s="17" t="inlineStr"/>
+      <c r="Q28" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_arup_amsterdam_science_industry_pm</t>
+        </is>
+      </c>
+      <c r="R28" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S28" s="17" t="inlineStr">
+        <is>
+          <t>Open solicitation (not a live vacancy), junior-friendly, same shape as the Design Manager open application. Real gap: fluent Dutch required, candidate has none — not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="21">
       <c r="A29" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Arup Amsterdam Tech/Data Centers PM row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2929,28 +2929,66 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="21">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="12" t="n"/>
-      <c r="J29" s="12" t="n"/>
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Arup</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Open Application – Project Management, Technology / Data Centers, Job AMS000092</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Amsterdam, NL</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr"/>
+      <c r="E29" s="17" t="inlineStr"/>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>https://jobs.arup.com/jobs/33870/other-jobs-matching/location-only</t>
+        </is>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I29" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J29" s="18" t="inlineStr"/>
       <c r="K29" s="14">
         <f>IF($H29="","",TODAY()-$H29)</f>
         <v/>
       </c>
-      <c r="L29" s="13" t="n"/>
-      <c r="M29" s="11" t="n"/>
-      <c r="N29" s="13" t="n"/>
-      <c r="O29" s="11" t="n"/>
-      <c r="P29" s="11" t="n"/>
-      <c r="Q29" s="11" t="n"/>
-      <c r="R29" s="12" t="n"/>
-      <c r="S29" s="11" t="n"/>
+      <c r="L29" s="19" t="inlineStr"/>
+      <c r="M29" s="17" t="inlineStr"/>
+      <c r="N29" s="19" t="inlineStr"/>
+      <c r="O29" s="17" t="inlineStr"/>
+      <c r="P29" s="17" t="inlineStr"/>
+      <c r="Q29" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_arup_amsterdam_tech_datacenters_pm</t>
+        </is>
+      </c>
+      <c r="R29" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S29" s="17" t="inlineStr">
+        <is>
+          <t>Third Arup Amsterdam open application (open solicitation, not a live vacancy), junior-friendly. Real gap: fluent Dutch required, candidate has none — not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="21">
       <c r="A30" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Building Physics Consultant row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -2991,28 +2991,78 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="21">
-      <c r="A30" s="11" t="n"/>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="11" t="n"/>
-      <c r="F30" s="11" t="n"/>
-      <c r="G30" s="11" t="n"/>
-      <c r="H30" s="13" t="n"/>
-      <c r="I30" s="12" t="n"/>
-      <c r="J30" s="12" t="n"/>
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Junior Building Physics Consultant – Fire, Environment &amp; Building Physics</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr"/>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66955</t>
+        </is>
+      </c>
+      <c r="H30" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J30" s="18" t="inlineStr"/>
       <c r="K30" s="14">
         <f>IF($H30="","",TODAY()-$H30)</f>
         <v/>
       </c>
-      <c r="L30" s="13" t="n"/>
-      <c r="M30" s="11" t="n"/>
-      <c r="N30" s="13" t="n"/>
-      <c r="O30" s="11" t="n"/>
-      <c r="P30" s="11" t="n"/>
-      <c r="Q30" s="11" t="n"/>
-      <c r="R30" s="12" t="n"/>
-      <c r="S30" s="11" t="n"/>
+      <c r="L30" s="19" t="inlineStr"/>
+      <c r="M30" s="17" t="inlineStr"/>
+      <c r="N30" s="19" t="inlineStr"/>
+      <c r="O30" s="17" t="inlineStr">
+        <is>
+          <t>Bas Peeters</t>
+        </is>
+      </c>
+      <c r="P30" s="17" t="inlineStr">
+        <is>
+          <t>bas.peeters@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q30" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_bas_peeters</t>
+        </is>
+      </c>
+      <c r="R30" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S30" s="17" t="inlineStr">
+        <is>
+          <t>Real domain mismatch — no daylight/energy/acoustics/fire-safety background at all (different specialization than BIM). Fluent Dutch also required. Applied anyway per explicit user instruction; leans on energy-management coursework + adaptability, gaps not disclosed.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="21">
       <c r="A31" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Fire Safety Advisor row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3065,28 +3065,82 @@
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="21">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="12" t="n"/>
-      <c r="E31" s="11" t="n"/>
-      <c r="F31" s="11" t="n"/>
-      <c r="G31" s="11" t="n"/>
-      <c r="H31" s="13" t="n"/>
-      <c r="I31" s="12" t="n"/>
-      <c r="J31" s="12" t="n"/>
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Junior Fire Safety Advisor – Fire, Environment &amp; Building Physics</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>Venlo/Eindhoven, NL</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,100/month</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G31" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66956</t>
+        </is>
+      </c>
+      <c r="H31" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I31" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J31" s="18" t="inlineStr"/>
       <c r="K31" s="14">
         <f>IF($H31="","",TODAY()-$H31)</f>
         <v/>
       </c>
-      <c r="L31" s="13" t="n"/>
-      <c r="M31" s="11" t="n"/>
-      <c r="N31" s="13" t="n"/>
-      <c r="O31" s="11" t="n"/>
-      <c r="P31" s="11" t="n"/>
-      <c r="Q31" s="11" t="n"/>
-      <c r="R31" s="12" t="n"/>
-      <c r="S31" s="11" t="n"/>
+      <c r="L31" s="19" t="inlineStr"/>
+      <c r="M31" s="17" t="inlineStr"/>
+      <c r="N31" s="19" t="inlineStr"/>
+      <c r="O31" s="17" t="inlineStr">
+        <is>
+          <t>Bas Peeters</t>
+        </is>
+      </c>
+      <c r="P31" s="17" t="inlineStr">
+        <is>
+          <t>bas.peeters@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q31" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_fire_safety_peeters</t>
+        </is>
+      </c>
+      <c r="R31" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S31" s="17" t="inlineStr">
+        <is>
+          <t>Same team/manager as the Building Physics Consultant posting; real domain gap (no fire-safety background) plus fluent Dutch required. Applied anyway per established preference for this team; gaps not disclosed.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="21">
       <c r="A32" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Advisor Cultural Engineering row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3143,28 +3143,82 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="21">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="11" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="11" t="n"/>
-      <c r="G32" s="11" t="n"/>
-      <c r="H32" s="13" t="n"/>
-      <c r="I32" s="12" t="n"/>
-      <c r="J32" s="12" t="n"/>
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Junior Advisor Cultural Engineering – Environmental and Cultural Engineering Research</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Eindhoven, NL</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66857</t>
+        </is>
+      </c>
+      <c r="H32" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J32" s="18" t="inlineStr"/>
       <c r="K32" s="14">
         <f>IF($H32="","",TODAY()-$H32)</f>
         <v/>
       </c>
-      <c r="L32" s="13" t="n"/>
-      <c r="M32" s="11" t="n"/>
-      <c r="N32" s="13" t="n"/>
-      <c r="O32" s="11" t="n"/>
-      <c r="P32" s="11" t="n"/>
-      <c r="Q32" s="11" t="n"/>
-      <c r="R32" s="12" t="n"/>
-      <c r="S32" s="11" t="n"/>
+      <c r="L32" s="19" t="inlineStr"/>
+      <c r="M32" s="17" t="inlineStr"/>
+      <c r="N32" s="19" t="inlineStr"/>
+      <c r="O32" s="17" t="inlineStr">
+        <is>
+          <t>Jules Rutten</t>
+        </is>
+      </c>
+      <c r="P32" s="17" t="inlineStr">
+        <is>
+          <t>jules.rutten@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q32" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_jules_rutten</t>
+        </is>
+      </c>
+      <c r="R32" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S32" s="17" t="inlineStr">
+        <is>
+          <t>Genuine domain fit via real hydrology/water-resources coursework (AutoCAD, HEC-HMS, HEC-RAS) — better fit than the Building Physics/Fire Safety Sweco roles. Dutch C1 required, not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="21">
       <c r="A33" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Architectural BIM Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3221,28 +3221,78 @@
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="21">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="12" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
-      <c r="H33" s="13" t="n"/>
-      <c r="I33" s="12" t="n"/>
-      <c r="J33" s="12" t="n"/>
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Architectural BIM Engineer – Logistics and Business Accommodation</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>De Bilt/Eindhoven/The Hague, NL</t>
+        </is>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,750-4,250/month</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66747</t>
+        </is>
+      </c>
+      <c r="H33" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I33" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J33" s="18" t="inlineStr"/>
       <c r="K33" s="14">
         <f>IF($H33="","",TODAY()-$H33)</f>
         <v/>
       </c>
-      <c r="L33" s="13" t="n"/>
-      <c r="M33" s="11" t="n"/>
-      <c r="N33" s="13" t="n"/>
-      <c r="O33" s="11" t="n"/>
-      <c r="P33" s="11" t="n"/>
-      <c r="Q33" s="11" t="n"/>
-      <c r="R33" s="12" t="n"/>
-      <c r="S33" s="11" t="n"/>
+      <c r="L33" s="19" t="inlineStr"/>
+      <c r="M33" s="17" t="inlineStr"/>
+      <c r="N33" s="19" t="inlineStr"/>
+      <c r="O33" s="17" t="inlineStr">
+        <is>
+          <t>Eric Thoma</t>
+        </is>
+      </c>
+      <c r="P33" s="17" t="inlineStr"/>
+      <c r="Q33" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_eric_thoma</t>
+        </is>
+      </c>
+      <c r="R33" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S33" s="17" t="inlineStr">
+        <is>
+          <t>Strong direct BIM match — Revit + multidisciplinary coordination maps closely onto the Guimarães project. Real gaps: 2 years experience, fluent Dutch — not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="21">
       <c r="A34" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Urban Planning Advisor row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3295,28 +3295,82 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="21">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="11" t="n"/>
-      <c r="C34" s="11" t="n"/>
-      <c r="D34" s="12" t="n"/>
-      <c r="E34" s="11" t="n"/>
-      <c r="F34" s="11" t="n"/>
-      <c r="G34" s="11" t="n"/>
-      <c r="H34" s="13" t="n"/>
-      <c r="I34" s="12" t="n"/>
-      <c r="J34" s="12" t="n"/>
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Urban Planning Advisor – Urban Projects South (Spatial Development)</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>Kapelle/Middelburg, NL</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,600-4,300/month</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66743</t>
+        </is>
+      </c>
+      <c r="H34" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I34" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J34" s="18" t="inlineStr"/>
       <c r="K34" s="14">
         <f>IF($H34="","",TODAY()-$H34)</f>
         <v/>
       </c>
-      <c r="L34" s="13" t="n"/>
-      <c r="M34" s="11" t="n"/>
-      <c r="N34" s="13" t="n"/>
-      <c r="O34" s="11" t="n"/>
-      <c r="P34" s="11" t="n"/>
-      <c r="Q34" s="11" t="n"/>
-      <c r="R34" s="12" t="n"/>
-      <c r="S34" s="11" t="n"/>
+      <c r="L34" s="19" t="inlineStr"/>
+      <c r="M34" s="17" t="inlineStr"/>
+      <c r="N34" s="19" t="inlineStr"/>
+      <c r="O34" s="17" t="inlineStr">
+        <is>
+          <t>Marik Waterman</t>
+        </is>
+      </c>
+      <c r="P34" s="17" t="inlineStr">
+        <is>
+          <t>marik.waterman@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q34" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_marik_waterman</t>
+        </is>
+      </c>
+      <c r="R34" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S34" s="17" t="inlineStr">
+        <is>
+          <t>Surfaced real urban planning coursework (previously untracked). Explicit ask for digitalization/AI experience is a genuine strength. No Dutch requirement listed. 2 years experience gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="21">
       <c r="A35" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Transport Pipeline Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3373,28 +3373,82 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="21">
-      <c r="A35" s="11" t="n"/>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="11" t="n"/>
-      <c r="G35" s="11" t="n"/>
-      <c r="H35" s="13" t="n"/>
-      <c r="I35" s="12" t="n"/>
-      <c r="J35" s="12" t="n"/>
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Transport Pipeline Engineer – Water</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>De Bilt, NL</t>
+        </is>
+      </c>
+      <c r="D35" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,600-4,300/month</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66744</t>
+        </is>
+      </c>
+      <c r="H35" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I35" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J35" s="18" t="inlineStr"/>
       <c r="K35" s="14">
         <f>IF($H35="","",TODAY()-$H35)</f>
         <v/>
       </c>
-      <c r="L35" s="13" t="n"/>
-      <c r="M35" s="11" t="n"/>
-      <c r="N35" s="13" t="n"/>
-      <c r="O35" s="11" t="n"/>
-      <c r="P35" s="11" t="n"/>
-      <c r="Q35" s="11" t="n"/>
-      <c r="R35" s="12" t="n"/>
-      <c r="S35" s="11" t="n"/>
+      <c r="L35" s="19" t="inlineStr"/>
+      <c r="M35" s="17" t="inlineStr"/>
+      <c r="N35" s="19" t="inlineStr"/>
+      <c r="O35" s="17" t="inlineStr">
+        <is>
+          <t>John Driessen</t>
+        </is>
+      </c>
+      <c r="P35" s="17" t="inlineStr">
+        <is>
+          <t>john.driessen@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q35" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_john_driessen</t>
+        </is>
+      </c>
+      <c r="R35" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S35" s="17" t="inlineStr">
+        <is>
+          <t>Genuine domain fit via real AutoCAD/ArcGIS/hydrology coursework, matching the posting’s explicit software asks. 1-3 years experience and Dutch C1 gaps not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="21">
       <c r="A36" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Construction PM Logistics row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3451,28 +3451,78 @@
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="21">
-      <c r="A36" s="11" t="n"/>
-      <c r="B36" s="11" t="n"/>
-      <c r="C36" s="11" t="n"/>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="11" t="n"/>
-      <c r="F36" s="11" t="n"/>
-      <c r="G36" s="11" t="n"/>
-      <c r="H36" s="13" t="n"/>
-      <c r="I36" s="12" t="n"/>
-      <c r="J36" s="12" t="n"/>
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Junior Construction Project Manager – Logistics and Business Accommodation</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>De Bilt/Amsterdam, NL</t>
+        </is>
+      </c>
+      <c r="D36" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,500-4,500/month</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G36" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66706</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I36" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J36" s="18" t="inlineStr"/>
       <c r="K36" s="14">
         <f>IF($H36="","",TODAY()-$H36)</f>
         <v/>
       </c>
-      <c r="L36" s="13" t="n"/>
-      <c r="M36" s="11" t="n"/>
-      <c r="N36" s="13" t="n"/>
-      <c r="O36" s="11" t="n"/>
-      <c r="P36" s="11" t="n"/>
-      <c r="Q36" s="11" t="n"/>
-      <c r="R36" s="12" t="n"/>
-      <c r="S36" s="11" t="n"/>
+      <c r="L36" s="19" t="inlineStr"/>
+      <c r="M36" s="17" t="inlineStr"/>
+      <c r="N36" s="19" t="inlineStr"/>
+      <c r="O36" s="17" t="inlineStr"/>
+      <c r="P36" s="17" t="inlineStr">
+        <is>
+          <t>lindsay.vanheugten@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q36" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_pm_logistics_thoma</t>
+        </is>
+      </c>
+      <c r="R36" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S36" s="17" t="inlineStr">
+        <is>
+          <t>Same team as the Architectural BIM Engineer application (Eric Thoma). 1-3 years experience and Dutch fluency gaps not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="21">
       <c r="A37" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Contract Management Advisor row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3525,28 +3525,82 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="21">
-      <c r="A37" s="11" t="n"/>
-      <c r="B37" s="11" t="n"/>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="12" t="n"/>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
-      <c r="H37" s="13" t="n"/>
-      <c r="I37" s="12" t="n"/>
-      <c r="J37" s="12" t="n"/>
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Junior Contract Management Advisor – Urban Projects</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>Rotterdam, NL</t>
+        </is>
+      </c>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,100/month</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66683</t>
+        </is>
+      </c>
+      <c r="H37" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I37" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J37" s="18" t="inlineStr"/>
       <c r="K37" s="14">
         <f>IF($H37="","",TODAY()-$H37)</f>
         <v/>
       </c>
-      <c r="L37" s="13" t="n"/>
-      <c r="M37" s="11" t="n"/>
-      <c r="N37" s="13" t="n"/>
-      <c r="O37" s="11" t="n"/>
-      <c r="P37" s="11" t="n"/>
-      <c r="Q37" s="11" t="n"/>
-      <c r="R37" s="12" t="n"/>
-      <c r="S37" s="11" t="n"/>
+      <c r="L37" s="19" t="inlineStr"/>
+      <c r="M37" s="17" t="inlineStr"/>
+      <c r="N37" s="19" t="inlineStr"/>
+      <c r="O37" s="17" t="inlineStr">
+        <is>
+          <t>Edyta Wisniewska</t>
+        </is>
+      </c>
+      <c r="P37" s="17" t="inlineStr">
+        <is>
+          <t>edyta.wisniewska@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q37" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_edyta_wisniewska</t>
+        </is>
+      </c>
+      <c r="R37" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S37" s="17" t="inlineStr">
+        <is>
+          <t>Strong match — graduate-entry framing, no Dutch requirement listed, and the FIDIC contract-review internship maps directly onto the role.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="21">
       <c r="A38" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Volantis Junior Project Manager row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3603,28 +3603,78 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="21">
-      <c r="A38" s="11" t="n"/>
-      <c r="B38" s="11" t="n"/>
-      <c r="C38" s="11" t="n"/>
-      <c r="D38" s="12" t="n"/>
-      <c r="E38" s="11" t="n"/>
-      <c r="F38" s="11" t="n"/>
-      <c r="G38" s="11" t="n"/>
-      <c r="H38" s="13" t="n"/>
-      <c r="I38" s="12" t="n"/>
-      <c r="J38" s="12" t="n"/>
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Project Manager – Volantis</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>Venlo/Eindhoven, NL</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr"/>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66682</t>
+        </is>
+      </c>
+      <c r="H38" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I38" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J38" s="18" t="inlineStr"/>
       <c r="K38" s="14">
         <f>IF($H38="","",TODAY()-$H38)</f>
         <v/>
       </c>
-      <c r="L38" s="13" t="n"/>
-      <c r="M38" s="11" t="n"/>
-      <c r="N38" s="13" t="n"/>
-      <c r="O38" s="11" t="n"/>
-      <c r="P38" s="11" t="n"/>
-      <c r="Q38" s="11" t="n"/>
-      <c r="R38" s="12" t="n"/>
-      <c r="S38" s="11" t="n"/>
+      <c r="L38" s="19" t="inlineStr"/>
+      <c r="M38" s="17" t="inlineStr"/>
+      <c r="N38" s="19" t="inlineStr"/>
+      <c r="O38" s="17" t="inlineStr">
+        <is>
+          <t>Pim Uiting</t>
+        </is>
+      </c>
+      <c r="P38" s="17" t="inlineStr">
+        <is>
+          <t>pim.uiting@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q38" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_volantis_pim_uiting</t>
+        </is>
+      </c>
+      <c r="R38" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S38" s="17" t="inlineStr">
+        <is>
+          <t>Graduate-friendly ("starters also welcome"). Fluent Dutch and English required, not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="21">
       <c r="A39" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Soil Consultant row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3677,28 +3677,82 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="21">
-      <c r="A39" s="11" t="n"/>
-      <c r="B39" s="11" t="n"/>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="12" t="n"/>
-      <c r="E39" s="11" t="n"/>
-      <c r="F39" s="11" t="n"/>
-      <c r="G39" s="11" t="n"/>
-      <c r="H39" s="13" t="n"/>
-      <c r="I39" s="12" t="n"/>
-      <c r="J39" s="12" t="n"/>
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Junior Soil Consultant – Environmental Consultancy</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>Groningen, NL</t>
+        </is>
+      </c>
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,100/month</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66601</t>
+        </is>
+      </c>
+      <c r="H39" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I39" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J39" s="18" t="inlineStr"/>
       <c r="K39" s="14">
         <f>IF($H39="","",TODAY()-$H39)</f>
         <v/>
       </c>
-      <c r="L39" s="13" t="n"/>
-      <c r="M39" s="11" t="n"/>
-      <c r="N39" s="13" t="n"/>
-      <c r="O39" s="11" t="n"/>
-      <c r="P39" s="11" t="n"/>
-      <c r="Q39" s="11" t="n"/>
-      <c r="R39" s="12" t="n"/>
-      <c r="S39" s="11" t="n"/>
+      <c r="L39" s="19" t="inlineStr"/>
+      <c r="M39" s="17" t="inlineStr"/>
+      <c r="N39" s="19" t="inlineStr"/>
+      <c r="O39" s="17" t="inlineStr">
+        <is>
+          <t>Mariska Moyaert</t>
+        </is>
+      </c>
+      <c r="P39" s="17" t="inlineStr">
+        <is>
+          <t>mariska.moyaert@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q39" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_mariska_moyaert</t>
+        </is>
+      </c>
+      <c r="R39" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S39" s="17" t="inlineStr">
+        <is>
+          <t>Domain-adjacent fit via real hydrology/water-resources/GIS coursework. Recent graduates explicitly welcomed. Dutch gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="21">
       <c r="A40" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Fire Safety Advisor (de Vries) row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3755,28 +3755,82 @@
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="21">
-      <c r="A40" s="11" t="n"/>
-      <c r="B40" s="11" t="n"/>
-      <c r="C40" s="11" t="n"/>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="11" t="n"/>
-      <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
-      <c r="H40" s="13" t="n"/>
-      <c r="I40" s="12" t="n"/>
-      <c r="J40" s="12" t="n"/>
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>Junior Fire Safety Advisor – Fire Safety &amp; Simulations</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>Amsterdam/Venlo/De Bilt/Rotterdam/Eindhoven, NL</t>
+        </is>
+      </c>
+      <c r="D40" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=66548</t>
+        </is>
+      </c>
+      <c r="H40" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I40" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J40" s="18" t="inlineStr"/>
       <c r="K40" s="14">
         <f>IF($H40="","",TODAY()-$H40)</f>
         <v/>
       </c>
-      <c r="L40" s="13" t="n"/>
-      <c r="M40" s="11" t="n"/>
-      <c r="N40" s="13" t="n"/>
-      <c r="O40" s="11" t="n"/>
-      <c r="P40" s="11" t="n"/>
-      <c r="Q40" s="11" t="n"/>
-      <c r="R40" s="12" t="n"/>
-      <c r="S40" s="11" t="n"/>
+      <c r="L40" s="19" t="inlineStr"/>
+      <c r="M40" s="17" t="inlineStr"/>
+      <c r="N40" s="19" t="inlineStr"/>
+      <c r="O40" s="17" t="inlineStr">
+        <is>
+          <t>Bart de Vries</t>
+        </is>
+      </c>
+      <c r="P40" s="17" t="inlineStr">
+        <is>
+          <t>bart.devries@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q40" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_bart_de_vries</t>
+        </is>
+      </c>
+      <c r="R40" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S40" s="17" t="inlineStr">
+        <is>
+          <t>Same domain gap as the earlier Peeters Fire Safety application (different team: Fire Safety &amp; Simulations). No fire-safety/CFD background. Dutch B2 minimum not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="21">
       <c r="A41" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Contract Writer Consultant row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3833,28 +3833,82 @@
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="21">
-      <c r="A41" s="11" t="n"/>
-      <c r="B41" s="11" t="n"/>
-      <c r="C41" s="11" t="n"/>
-      <c r="D41" s="12" t="n"/>
-      <c r="E41" s="11" t="n"/>
-      <c r="F41" s="11" t="n"/>
-      <c r="G41" s="11" t="n"/>
-      <c r="H41" s="13" t="n"/>
-      <c r="I41" s="12" t="n"/>
-      <c r="J41" s="12" t="n"/>
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Junior Contract Writer Consultant – Civil Engineering (Northern Netherlands)</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>Groningen/Leeuwarden, NL</t>
+        </is>
+      </c>
+      <c r="D41" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,100/month</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G41" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=65625</t>
+        </is>
+      </c>
+      <c r="H41" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I41" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J41" s="18" t="inlineStr"/>
       <c r="K41" s="14">
         <f>IF($H41="","",TODAY()-$H41)</f>
         <v/>
       </c>
-      <c r="L41" s="13" t="n"/>
-      <c r="M41" s="11" t="n"/>
-      <c r="N41" s="13" t="n"/>
-      <c r="O41" s="11" t="n"/>
-      <c r="P41" s="11" t="n"/>
-      <c r="Q41" s="11" t="n"/>
-      <c r="R41" s="12" t="n"/>
-      <c r="S41" s="11" t="n"/>
+      <c r="L41" s="19" t="inlineStr"/>
+      <c r="M41" s="17" t="inlineStr"/>
+      <c r="N41" s="19" t="inlineStr"/>
+      <c r="O41" s="17" t="inlineStr">
+        <is>
+          <t>Annemarie Rook / Kees van der Molen</t>
+        </is>
+      </c>
+      <c r="P41" s="17" t="inlineStr">
+        <is>
+          <t>annemarie.rook@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q41" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_contract_writer_groningen</t>
+        </is>
+      </c>
+      <c r="R41" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S41" s="17" t="inlineStr">
+        <is>
+          <t>Strong match — explicit digitalization/AI requirement is a genuine strength, plus the FIDIC contract-review internship. No Dutch requirement listed.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="21">
       <c r="A42" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Civil Engineering PM (Urban Projects) row to tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3911,28 +3911,82 @@
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="21">
-      <c r="A42" s="11" t="n"/>
-      <c r="B42" s="11" t="n"/>
-      <c r="C42" s="11" t="n"/>
-      <c r="D42" s="12" t="n"/>
-      <c r="E42" s="11" t="n"/>
-      <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
-      <c r="H42" s="13" t="n"/>
-      <c r="I42" s="12" t="n"/>
-      <c r="J42" s="12" t="n"/>
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Junior Civil Engineering Project Manager – Urban Projects</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>De Bilt, NL</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F42" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G42" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=65797</t>
+        </is>
+      </c>
+      <c r="H42" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I42" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J42" s="18" t="inlineStr"/>
       <c r="K42" s="14">
         <f>IF($H42="","",TODAY()-$H42)</f>
         <v/>
       </c>
-      <c r="L42" s="13" t="n"/>
-      <c r="M42" s="11" t="n"/>
-      <c r="N42" s="13" t="n"/>
-      <c r="O42" s="11" t="n"/>
-      <c r="P42" s="11" t="n"/>
-      <c r="Q42" s="11" t="n"/>
-      <c r="R42" s="12" t="n"/>
-      <c r="S42" s="11" t="n"/>
+      <c r="L42" s="19" t="inlineStr"/>
+      <c r="M42" s="17" t="inlineStr"/>
+      <c r="N42" s="19" t="inlineStr"/>
+      <c r="O42" s="17" t="inlineStr">
+        <is>
+          <t>Bart Witte</t>
+        </is>
+      </c>
+      <c r="P42" s="17" t="inlineStr">
+        <is>
+          <t>bart.witte@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q42" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_pm_urban_projects_witte</t>
+        </is>
+      </c>
+      <c r="R42" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S42" s="17" t="inlineStr">
+        <is>
+          <t>Second application involving Bart Witte as contact (previously Junior BIM Modeller Alkmaar). Fluent Dutch required, not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="21">
       <c r="A43" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Road Engineering Consultant row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -3989,28 +3989,82 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="21">
-      <c r="A43" s="11" t="n"/>
-      <c r="B43" s="11" t="n"/>
-      <c r="C43" s="11" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="11" t="n"/>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="13" t="n"/>
-      <c r="I43" s="12" t="n"/>
-      <c r="J43" s="12" t="n"/>
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>Junior Road Engineering Consultant – Living Environment</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>Alkmaar, NL</t>
+        </is>
+      </c>
+      <c r="D43" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F43" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=64592</t>
+        </is>
+      </c>
+      <c r="H43" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I43" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J43" s="18" t="inlineStr"/>
       <c r="K43" s="14">
         <f>IF($H43="","",TODAY()-$H43)</f>
         <v/>
       </c>
-      <c r="L43" s="13" t="n"/>
-      <c r="M43" s="11" t="n"/>
-      <c r="N43" s="13" t="n"/>
-      <c r="O43" s="11" t="n"/>
-      <c r="P43" s="11" t="n"/>
-      <c r="Q43" s="11" t="n"/>
-      <c r="R43" s="12" t="n"/>
-      <c r="S43" s="11" t="n"/>
+      <c r="L43" s="19" t="inlineStr"/>
+      <c r="M43" s="17" t="inlineStr"/>
+      <c r="N43" s="19" t="inlineStr"/>
+      <c r="O43" s="17" t="inlineStr">
+        <is>
+          <t>Bart Witte</t>
+        </is>
+      </c>
+      <c r="P43" s="17" t="inlineStr">
+        <is>
+          <t>bart.witte@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q43" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_road_engineering_witte</t>
+        </is>
+      </c>
+      <c r="R43" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S43" s="17" t="inlineStr">
+        <is>
+          <t>Third application to Bart Witte (confirmed with user before proceeding). No specific technical software gap; Dutch C1 required, not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="21">
       <c r="A44" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Structural Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4067,28 +4067,82 @@
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="21">
-      <c r="A44" s="11" t="n"/>
-      <c r="B44" s="11" t="n"/>
-      <c r="C44" s="11" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="11" t="n"/>
-      <c r="F44" s="11" t="n"/>
-      <c r="G44" s="11" t="n"/>
-      <c r="H44" s="13" t="n"/>
-      <c r="I44" s="12" t="n"/>
-      <c r="J44" s="12" t="n"/>
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="inlineStr">
+        <is>
+          <t>Junior Structural Engineer – Engineering &amp; Consultancy Construction</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>Groningen/Zwolle, NL</t>
+        </is>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F44" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G44" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=63877</t>
+        </is>
+      </c>
+      <c r="H44" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I44" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J44" s="18" t="inlineStr"/>
       <c r="K44" s="14">
         <f>IF($H44="","",TODAY()-$H44)</f>
         <v/>
       </c>
-      <c r="L44" s="13" t="n"/>
-      <c r="M44" s="11" t="n"/>
-      <c r="N44" s="13" t="n"/>
-      <c r="O44" s="11" t="n"/>
-      <c r="P44" s="11" t="n"/>
-      <c r="Q44" s="11" t="n"/>
-      <c r="R44" s="12" t="n"/>
-      <c r="S44" s="11" t="n"/>
+      <c r="L44" s="19" t="inlineStr"/>
+      <c r="M44" s="17" t="inlineStr"/>
+      <c r="N44" s="19" t="inlineStr"/>
+      <c r="O44" s="17" t="inlineStr">
+        <is>
+          <t>Sjaak Schreuder</t>
+        </is>
+      </c>
+      <c r="P44" s="17" t="inlineStr">
+        <is>
+          <t>sjaak.schreuder@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q44" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_sjaak_schreuder</t>
+        </is>
+      </c>
+      <c r="R44" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S44" s="17" t="inlineStr">
+        <is>
+          <t>Same domain gap as the Arup Bridge Engineer role — requires structural calculations and Scia/Technosoft, neither of which the candidate has. Dutch gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="21">
       <c r="A45" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior BIM Modeler Civil Engineering row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4145,28 +4145,82 @@
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="21">
-      <c r="A45" s="11" t="n"/>
-      <c r="B45" s="11" t="n"/>
-      <c r="C45" s="11" t="n"/>
-      <c r="D45" s="12" t="n"/>
-      <c r="E45" s="11" t="n"/>
-      <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
-      <c r="H45" s="13" t="n"/>
-      <c r="I45" s="12" t="n"/>
-      <c r="J45" s="12" t="n"/>
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>Junior BIM Modeler Civil Engineering – Urban Projects</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>De Bilt, NL</t>
+        </is>
+      </c>
+      <c r="D45" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F45" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=62537</t>
+        </is>
+      </c>
+      <c r="H45" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I45" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J45" s="18" t="inlineStr"/>
       <c r="K45" s="14">
         <f>IF($H45="","",TODAY()-$H45)</f>
         <v/>
       </c>
-      <c r="L45" s="13" t="n"/>
-      <c r="M45" s="11" t="n"/>
-      <c r="N45" s="13" t="n"/>
-      <c r="O45" s="11" t="n"/>
-      <c r="P45" s="11" t="n"/>
-      <c r="Q45" s="11" t="n"/>
-      <c r="R45" s="12" t="n"/>
-      <c r="S45" s="11" t="n"/>
+      <c r="L45" s="19" t="inlineStr"/>
+      <c r="M45" s="17" t="inlineStr"/>
+      <c r="N45" s="19" t="inlineStr"/>
+      <c r="O45" s="17" t="inlineStr">
+        <is>
+          <t>Robin Bree</t>
+        </is>
+      </c>
+      <c r="P45" s="17" t="inlineStr">
+        <is>
+          <t>lindsay.vanheugten@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q45" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_robin_bree</t>
+        </is>
+      </c>
+      <c r="R45" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S45" s="17" t="inlineStr">
+        <is>
+          <t>Strong direct match (Revit/Civil 3D modelling role). Dutch gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="21">
       <c r="A46" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco (Junior) Structural Modeler row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4223,28 +4223,82 @@
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="21">
-      <c r="A46" s="11" t="n"/>
-      <c r="B46" s="11" t="n"/>
-      <c r="C46" s="11" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="11" t="n"/>
-      <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
-      <c r="H46" s="13" t="n"/>
-      <c r="I46" s="12" t="n"/>
-      <c r="J46" s="12" t="n"/>
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Structural Modeler – Engineering &amp; Consultancy Construction</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>Groningen, NL</t>
+        </is>
+      </c>
+      <c r="D46" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F46" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G46" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=62445</t>
+        </is>
+      </c>
+      <c r="H46" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I46" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J46" s="18" t="inlineStr"/>
       <c r="K46" s="14">
         <f>IF($H46="","",TODAY()-$H46)</f>
         <v/>
       </c>
-      <c r="L46" s="13" t="n"/>
-      <c r="M46" s="11" t="n"/>
-      <c r="N46" s="13" t="n"/>
-      <c r="O46" s="11" t="n"/>
-      <c r="P46" s="11" t="n"/>
-      <c r="Q46" s="11" t="n"/>
-      <c r="R46" s="12" t="n"/>
-      <c r="S46" s="11" t="n"/>
+      <c r="L46" s="19" t="inlineStr"/>
+      <c r="M46" s="17" t="inlineStr"/>
+      <c r="N46" s="19" t="inlineStr"/>
+      <c r="O46" s="17" t="inlineStr">
+        <is>
+          <t>Jasper Pouls</t>
+        </is>
+      </c>
+      <c r="P46" s="17" t="inlineStr">
+        <is>
+          <t>jasper.pouls@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q46" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_jasper_pouls</t>
+        </is>
+      </c>
+      <c r="R46" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S46" s="17" t="inlineStr">
+        <is>
+          <t>Good direct match (Revit-based modelling role, not pure structural calculation). Dutch gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="21">
       <c r="A47" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Civil Designer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4301,28 +4301,82 @@
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="21">
-      <c r="A47" s="11" t="n"/>
-      <c r="B47" s="11" t="n"/>
-      <c r="C47" s="11" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="11" t="n"/>
-      <c r="F47" s="11" t="n"/>
-      <c r="G47" s="11" t="n"/>
-      <c r="H47" s="13" t="n"/>
-      <c r="I47" s="12" t="n"/>
-      <c r="J47" s="12" t="n"/>
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>Junior Civil Designer – Integrated Infrastructure Design</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>Amsterdam/De Bilt/Rotterdam/Alkmaar, NL</t>
+        </is>
+      </c>
+      <c r="D47" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=61191</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I47" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J47" s="18" t="inlineStr"/>
       <c r="K47" s="14">
         <f>IF($H47="","",TODAY()-$H47)</f>
         <v/>
       </c>
-      <c r="L47" s="13" t="n"/>
-      <c r="M47" s="11" t="n"/>
-      <c r="N47" s="13" t="n"/>
-      <c r="O47" s="11" t="n"/>
-      <c r="P47" s="11" t="n"/>
-      <c r="Q47" s="11" t="n"/>
-      <c r="R47" s="12" t="n"/>
-      <c r="S47" s="11" t="n"/>
+      <c r="L47" s="19" t="inlineStr"/>
+      <c r="M47" s="17" t="inlineStr"/>
+      <c r="N47" s="19" t="inlineStr"/>
+      <c r="O47" s="17" t="inlineStr">
+        <is>
+          <t>Peter Koelman</t>
+        </is>
+      </c>
+      <c r="P47" s="17" t="inlineStr">
+        <is>
+          <t>peter.koelman@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q47" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_peter_koelman</t>
+        </is>
+      </c>
+      <c r="R47" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S47" s="17" t="inlineStr">
+        <is>
+          <t>Strong match — no Dutch requirement listed, explicit AI/digitalization emphasis is a genuine strength.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="21">
       <c r="A48" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Civil Engineering Project Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4379,28 +4379,82 @@
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="21">
-      <c r="A48" s="11" t="n"/>
-      <c r="B48" s="11" t="n"/>
-      <c r="C48" s="11" t="n"/>
-      <c r="D48" s="12" t="n"/>
-      <c r="E48" s="11" t="n"/>
-      <c r="F48" s="11" t="n"/>
-      <c r="G48" s="11" t="n"/>
-      <c r="H48" s="13" t="n"/>
-      <c r="I48" s="12" t="n"/>
-      <c r="J48" s="12" t="n"/>
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Civil Engineering Project Engineer – Infrastructure</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Zwolle, NL</t>
+        </is>
+      </c>
+      <c r="D48" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F48" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G48" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=55138</t>
+        </is>
+      </c>
+      <c r="H48" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I48" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J48" s="18" t="inlineStr"/>
       <c r="K48" s="14">
         <f>IF($H48="","",TODAY()-$H48)</f>
         <v/>
       </c>
-      <c r="L48" s="13" t="n"/>
-      <c r="M48" s="11" t="n"/>
-      <c r="N48" s="13" t="n"/>
-      <c r="O48" s="11" t="n"/>
-      <c r="P48" s="11" t="n"/>
-      <c r="Q48" s="11" t="n"/>
-      <c r="R48" s="12" t="n"/>
-      <c r="S48" s="11" t="n"/>
+      <c r="L48" s="19" t="inlineStr"/>
+      <c r="M48" s="17" t="inlineStr"/>
+      <c r="N48" s="19" t="inlineStr"/>
+      <c r="O48" s="17" t="inlineStr">
+        <is>
+          <t>Jeroen van de Uitvlugt</t>
+        </is>
+      </c>
+      <c r="P48" s="17" t="inlineStr">
+        <is>
+          <t>jeroen.vandeuitvlugt@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q48" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_jeroen_uitvlugt</t>
+        </is>
+      </c>
+      <c r="R48" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S48" s="17" t="inlineStr">
+        <is>
+          <t>Strong match — no Dutch requirement listed; AutoCAD, cost estimation and FIDIC contract-review experience all genuine strengths.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="21">
       <c r="A49" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Road Management Advisor row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4457,28 +4457,78 @@
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="21">
-      <c r="A49" s="11" t="n"/>
-      <c r="B49" s="11" t="n"/>
-      <c r="C49" s="11" t="n"/>
-      <c r="D49" s="12" t="n"/>
-      <c r="E49" s="11" t="n"/>
-      <c r="F49" s="11" t="n"/>
-      <c r="G49" s="11" t="n"/>
-      <c r="H49" s="13" t="n"/>
-      <c r="I49" s="12" t="n"/>
-      <c r="J49" s="12" t="n"/>
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
+        <is>
+          <t>Junior Road Management Advisor</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>Multiple NL offices (Middelburg/Groningen/Arnhem/Leeuwarden/De Bilt/Rotterdam/Alkmaar/Eindhoven/Amsterdam)</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr"/>
+      <c r="F49" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G49" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=52972</t>
+        </is>
+      </c>
+      <c r="H49" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I49" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J49" s="18" t="inlineStr"/>
       <c r="K49" s="14">
         <f>IF($H49="","",TODAY()-$H49)</f>
         <v/>
       </c>
-      <c r="L49" s="13" t="n"/>
-      <c r="M49" s="11" t="n"/>
-      <c r="N49" s="13" t="n"/>
-      <c r="O49" s="11" t="n"/>
-      <c r="P49" s="11" t="n"/>
-      <c r="Q49" s="11" t="n"/>
-      <c r="R49" s="12" t="n"/>
-      <c r="S49" s="11" t="n"/>
+      <c r="L49" s="19" t="inlineStr"/>
+      <c r="M49" s="17" t="inlineStr"/>
+      <c r="N49" s="19" t="inlineStr"/>
+      <c r="O49" s="17" t="inlineStr">
+        <is>
+          <t>Rob Krom</t>
+        </is>
+      </c>
+      <c r="P49" s="17" t="inlineStr">
+        <is>
+          <t>rob.krom@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q49" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_rob_krom</t>
+        </is>
+      </c>
+      <c r="R49" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S49" s="17" t="inlineStr">
+        <is>
+          <t>Strong match — no Dutch requirement listed; GIS (ArcGIS) and explicit AI/digitalization asks are both genuine strengths.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="21">
       <c r="A50" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Hydraulic Engineering Design Manager row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4531,28 +4531,82 @@
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="21">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="11" t="n"/>
-      <c r="D50" s="12" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="11" t="n"/>
-      <c r="H50" s="13" t="n"/>
-      <c r="I50" s="12" t="n"/>
-      <c r="J50" s="12" t="n"/>
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Hydraulic Engineering Design Manager – Structural Hydraulic Engineering</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>De Bilt/Rotterdam/Amsterdam, NL</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>EUR 4,000-5,500/month</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G50" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=50518</t>
+        </is>
+      </c>
+      <c r="H50" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I50" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J50" s="18" t="inlineStr"/>
       <c r="K50" s="14">
         <f>IF($H50="","",TODAY()-$H50)</f>
         <v/>
       </c>
-      <c r="L50" s="13" t="n"/>
-      <c r="M50" s="11" t="n"/>
-      <c r="N50" s="13" t="n"/>
-      <c r="O50" s="11" t="n"/>
-      <c r="P50" s="11" t="n"/>
-      <c r="Q50" s="11" t="n"/>
-      <c r="R50" s="12" t="n"/>
-      <c r="S50" s="11" t="n"/>
+      <c r="L50" s="19" t="inlineStr"/>
+      <c r="M50" s="17" t="inlineStr"/>
+      <c r="N50" s="19" t="inlineStr"/>
+      <c r="O50" s="17" t="inlineStr">
+        <is>
+          <t>Jan Hein Poodt</t>
+        </is>
+      </c>
+      <c r="P50" s="17" t="inlineStr">
+        <is>
+          <t>jan-hein.poodt@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q50" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_jan_hein_poodt</t>
+        </is>
+      </c>
+      <c r="R50" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S50" s="17" t="inlineStr">
+        <is>
+          <t>Long-shot per user request — 5 years experience required despite "(Junior)" title, mid-level salary band. Good domain fit (hydrology/water resources coursework) but real seniority gap.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="21">
       <c r="A51" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Underground Infrastructure & Water row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4609,28 +4609,82 @@
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="21">
-      <c r="A51" s="11" t="n"/>
-      <c r="B51" s="11" t="n"/>
-      <c r="C51" s="11" t="n"/>
-      <c r="D51" s="12" t="n"/>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="11" t="n"/>
-      <c r="H51" s="13" t="n"/>
-      <c r="I51" s="12" t="n"/>
-      <c r="J51" s="12" t="n"/>
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Junior Advisor Underground Infrastructure &amp; Water</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>De Bilt, NL</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-3,766/month</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G51" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=47996</t>
+        </is>
+      </c>
+      <c r="H51" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I51" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J51" s="18" t="inlineStr"/>
       <c r="K51" s="14">
         <f>IF($H51="","",TODAY()-$H51)</f>
         <v/>
       </c>
-      <c r="L51" s="13" t="n"/>
-      <c r="M51" s="11" t="n"/>
-      <c r="N51" s="13" t="n"/>
-      <c r="O51" s="11" t="n"/>
-      <c r="P51" s="11" t="n"/>
-      <c r="Q51" s="11" t="n"/>
-      <c r="R51" s="12" t="n"/>
-      <c r="S51" s="11" t="n"/>
+      <c r="L51" s="19" t="inlineStr"/>
+      <c r="M51" s="17" t="inlineStr"/>
+      <c r="N51" s="19" t="inlineStr"/>
+      <c r="O51" s="17" t="inlineStr">
+        <is>
+          <t>John Driessen</t>
+        </is>
+      </c>
+      <c r="P51" s="17" t="inlineStr">
+        <is>
+          <t>john.driessen@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q51" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_underground_infra_driessen</t>
+        </is>
+      </c>
+      <c r="R51" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S51" s="17" t="inlineStr">
+        <is>
+          <t>Second application to John Driessen (previously Transport Pipeline Engineer). Strong match — GIS/data science/BIM explicitly named, no Dutch requirement listed, graduate-friendly.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="21">
       <c r="A52" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Structural Engineer Middelburg row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4687,28 +4687,82 @@
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="21">
-      <c r="A52" s="11" t="n"/>
-      <c r="B52" s="11" t="n"/>
-      <c r="C52" s="11" t="n"/>
-      <c r="D52" s="12" t="n"/>
-      <c r="E52" s="11" t="n"/>
-      <c r="F52" s="11" t="n"/>
-      <c r="G52" s="11" t="n"/>
-      <c r="H52" s="13" t="n"/>
-      <c r="I52" s="12" t="n"/>
-      <c r="J52" s="12" t="n"/>
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Structural Engineer – Engineering &amp; Consultancy Construction</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Middelburg, NL</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=53226</t>
+        </is>
+      </c>
+      <c r="H52" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I52" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J52" s="18" t="inlineStr"/>
       <c r="K52" s="14">
         <f>IF($H52="","",TODAY()-$H52)</f>
         <v/>
       </c>
-      <c r="L52" s="13" t="n"/>
-      <c r="M52" s="11" t="n"/>
-      <c r="N52" s="13" t="n"/>
-      <c r="O52" s="11" t="n"/>
-      <c r="P52" s="11" t="n"/>
-      <c r="Q52" s="11" t="n"/>
-      <c r="R52" s="12" t="n"/>
-      <c r="S52" s="11" t="n"/>
+      <c r="L52" s="19" t="inlineStr"/>
+      <c r="M52" s="17" t="inlineStr"/>
+      <c r="N52" s="19" t="inlineStr"/>
+      <c r="O52" s="17" t="inlineStr">
+        <is>
+          <t>Michel van Aert</t>
+        </is>
+      </c>
+      <c r="P52" s="17" t="inlineStr">
+        <is>
+          <t>michel.vanaert@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q52" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_michel_van_aert</t>
+        </is>
+      </c>
+      <c r="R52" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S52" s="17" t="inlineStr">
+        <is>
+          <t>Same shape as the Schreuder/Pouls structural roles (Revit-based modelling, different branch). Dutch gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="21">
       <c r="A53" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Junior Project Consultant row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4765,28 +4765,82 @@
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="21">
-      <c r="A53" s="11" t="n"/>
-      <c r="B53" s="11" t="n"/>
-      <c r="C53" s="11" t="n"/>
-      <c r="D53" s="12" t="n"/>
-      <c r="E53" s="11" t="n"/>
-      <c r="F53" s="11" t="n"/>
-      <c r="G53" s="11" t="n"/>
-      <c r="H53" s="13" t="n"/>
-      <c r="I53" s="12" t="n"/>
-      <c r="J53" s="12" t="n"/>
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Junior Project Consultant – Area Development</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>Arnhem, NL</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=39914</t>
+        </is>
+      </c>
+      <c r="H53" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I53" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J53" s="18" t="inlineStr"/>
       <c r="K53" s="14">
         <f>IF($H53="","",TODAY()-$H53)</f>
         <v/>
       </c>
-      <c r="L53" s="13" t="n"/>
-      <c r="M53" s="11" t="n"/>
-      <c r="N53" s="13" t="n"/>
-      <c r="O53" s="11" t="n"/>
-      <c r="P53" s="11" t="n"/>
-      <c r="Q53" s="11" t="n"/>
-      <c r="R53" s="12" t="n"/>
-      <c r="S53" s="11" t="n"/>
+      <c r="L53" s="19" t="inlineStr"/>
+      <c r="M53" s="17" t="inlineStr"/>
+      <c r="N53" s="19" t="inlineStr"/>
+      <c r="O53" s="17" t="inlineStr">
+        <is>
+          <t>Marcel Janssen</t>
+        </is>
+      </c>
+      <c r="P53" s="17" t="inlineStr">
+        <is>
+          <t>marcel.janssen@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q53" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_marcel_janssen</t>
+        </is>
+      </c>
+      <c r="R53" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S53" s="17" t="inlineStr">
+        <is>
+          <t>Good match — digitalization/AI explicitly a plus, civil engineering/land-water framing fits. Dutch gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="21">
       <c r="A54" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco (Junior) Civil Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4843,28 +4843,82 @@
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="21">
-      <c r="A54" s="11" t="n"/>
-      <c r="B54" s="11" t="n"/>
-      <c r="C54" s="11" t="n"/>
-      <c r="D54" s="12" t="n"/>
-      <c r="E54" s="11" t="n"/>
-      <c r="F54" s="11" t="n"/>
-      <c r="G54" s="11" t="n"/>
-      <c r="H54" s="13" t="n"/>
-      <c r="I54" s="12" t="n"/>
-      <c r="J54" s="12" t="n"/>
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) Civil Engineer – Engineering and Urban Projects</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>Multiple NL offices (Alkmaar/Amsterdam/Middelburg/Arnhem/Groningen/Zwolle/Leeuwarden/De Bilt)</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,442-4,000/month</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.nl/solliciteren/?vacancy=39949</t>
+        </is>
+      </c>
+      <c r="H54" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I54" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J54" s="18" t="inlineStr"/>
       <c r="K54" s="14">
         <f>IF($H54="","",TODAY()-$H54)</f>
         <v/>
       </c>
-      <c r="L54" s="13" t="n"/>
-      <c r="M54" s="11" t="n"/>
-      <c r="N54" s="13" t="n"/>
-      <c r="O54" s="11" t="n"/>
-      <c r="P54" s="11" t="n"/>
-      <c r="Q54" s="11" t="n"/>
-      <c r="R54" s="12" t="n"/>
-      <c r="S54" s="11" t="n"/>
+      <c r="L54" s="19" t="inlineStr"/>
+      <c r="M54" s="17" t="inlineStr"/>
+      <c r="N54" s="19" t="inlineStr"/>
+      <c r="O54" s="17" t="inlineStr">
+        <is>
+          <t>Robin Bree</t>
+        </is>
+      </c>
+      <c r="P54" s="17" t="inlineStr">
+        <is>
+          <t>lindsay.vanheugten@sweco.nl</t>
+        </is>
+      </c>
+      <c r="Q54" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_sweco_civil_engineer_bree</t>
+        </is>
+      </c>
+      <c r="R54" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S54" s="17" t="inlineStr">
+        <is>
+          <t>Second application to Robin Bree (previously BIM Modeler Civil Engineering). Strong overall match: AutoCAD, digitalization/AI, FIDIC contract review all genuine strengths.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="21">
       <c r="A55" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Denmark District Heating PM row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4921,28 +4921,66 @@
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="21">
-      <c r="A55" s="11" t="n"/>
-      <c r="B55" s="11" t="n"/>
-      <c r="C55" s="11" t="n"/>
-      <c r="D55" s="12" t="n"/>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="11" t="n"/>
-      <c r="G55" s="11" t="n"/>
-      <c r="H55" s="13" t="n"/>
-      <c r="I55" s="12" t="n"/>
-      <c r="J55" s="12" t="n"/>
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>Sweco Energi</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>Junior Project Manager – District Heating Projects</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>Greater Copenhagen / North Zealand, DK</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr"/>
+      <c r="E55" s="17" t="inlineStr"/>
+      <c r="F55" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>https://candidate.hr-manager.net/ApplicationInit.aspx?cid=87&amp;ProjectId=183677&amp;DepartmentId=2127&amp;SkipAdvertisement=true</t>
+        </is>
+      </c>
+      <c r="H55" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I55" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J55" s="18" t="inlineStr"/>
       <c r="K55" s="14">
         <f>IF($H55="","",TODAY()-$H55)</f>
         <v/>
       </c>
-      <c r="L55" s="13" t="n"/>
-      <c r="M55" s="11" t="n"/>
-      <c r="N55" s="13" t="n"/>
-      <c r="O55" s="11" t="n"/>
-      <c r="P55" s="11" t="n"/>
-      <c r="Q55" s="11" t="n"/>
-      <c r="R55" s="12" t="n"/>
-      <c r="S55" s="11" t="n"/>
+      <c r="L55" s="19" t="inlineStr"/>
+      <c r="M55" s="17" t="inlineStr"/>
+      <c r="N55" s="19" t="inlineStr"/>
+      <c r="O55" s="17" t="inlineStr"/>
+      <c r="P55" s="17" t="inlineStr"/>
+      <c r="Q55" s="17" t="inlineStr">
+        <is>
+          <t>denmark/2026_08_04_sweco_district_heating_pm</t>
+        </is>
+      </c>
+      <c r="R55" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S55" s="17" t="inlineStr">
+        <is>
+          <t>3 years experience required, not disclosed per updated default. No explicit language requirement listed. Leans on real energy-management coursework.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="21">
       <c r="A56" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Belgium Junior Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -4983,28 +4983,66 @@
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="21">
-      <c r="A56" s="11" t="n"/>
-      <c r="B56" s="11" t="n"/>
-      <c r="C56" s="11" t="n"/>
-      <c r="D56" s="12" t="n"/>
-      <c r="E56" s="11" t="n"/>
-      <c r="F56" s="11" t="n"/>
-      <c r="G56" s="11" t="n"/>
-      <c r="H56" s="13" t="n"/>
-      <c r="I56" s="12" t="n"/>
-      <c r="J56" s="12" t="n"/>
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>Junior Engineer (Req. 269)</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>Multiple BE/LU offices (Berchem/Gent/Brussels/Hasselt/Leuven and others)</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr"/>
+      <c r="F56" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="inlineStr"/>
+      <c r="H56" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I56" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J56" s="18" t="inlineStr"/>
       <c r="K56" s="14">
         <f>IF($H56="","",TODAY()-$H56)</f>
         <v/>
       </c>
-      <c r="L56" s="13" t="n"/>
-      <c r="M56" s="11" t="n"/>
-      <c r="N56" s="13" t="n"/>
-      <c r="O56" s="11" t="n"/>
-      <c r="P56" s="11" t="n"/>
-      <c r="Q56" s="11" t="n"/>
-      <c r="R56" s="12" t="n"/>
-      <c r="S56" s="11" t="n"/>
+      <c r="L56" s="19" t="inlineStr"/>
+      <c r="M56" s="17" t="inlineStr"/>
+      <c r="N56" s="19" t="inlineStr"/>
+      <c r="O56" s="17" t="inlineStr"/>
+      <c r="P56" s="17" t="inlineStr"/>
+      <c r="Q56" s="17" t="inlineStr">
+        <is>
+          <t>belgium/2026_08_04_sweco_junior_engineer</t>
+        </is>
+      </c>
+      <c r="R56" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S56" s="17" t="inlineStr">
+        <is>
+          <t>No language/software requirement listed, explicitly open to near-graduates. Excellent accessibility, strong AI/digitalization profile fits well.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="21">
       <c r="A57" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Belgium BIM Coordinator row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5045,28 +5045,66 @@
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="21">
-      <c r="A57" s="11" t="n"/>
-      <c r="B57" s="11" t="n"/>
-      <c r="C57" s="11" t="n"/>
-      <c r="D57" s="12" t="n"/>
-      <c r="E57" s="11" t="n"/>
-      <c r="F57" s="11" t="n"/>
-      <c r="G57" s="11" t="n"/>
-      <c r="H57" s="13" t="n"/>
-      <c r="I57" s="12" t="n"/>
-      <c r="J57" s="12" t="n"/>
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>BIM Coordinator (Req. 1359)</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>Antwerp, BE (also Ghent/Berchem/Brussels and others)</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr"/>
+      <c r="F57" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr"/>
+      <c r="H57" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I57" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J57" s="18" t="inlineStr"/>
       <c r="K57" s="14">
         <f>IF($H57="","",TODAY()-$H57)</f>
         <v/>
       </c>
-      <c r="L57" s="13" t="n"/>
-      <c r="M57" s="11" t="n"/>
-      <c r="N57" s="13" t="n"/>
-      <c r="O57" s="11" t="n"/>
-      <c r="P57" s="11" t="n"/>
-      <c r="Q57" s="11" t="n"/>
-      <c r="R57" s="12" t="n"/>
-      <c r="S57" s="11" t="n"/>
+      <c r="L57" s="19" t="inlineStr"/>
+      <c r="M57" s="17" t="inlineStr"/>
+      <c r="N57" s="19" t="inlineStr"/>
+      <c r="O57" s="17" t="inlineStr"/>
+      <c r="P57" s="17" t="inlineStr"/>
+      <c r="Q57" s="17" t="inlineStr">
+        <is>
+          <t>belgium/2026_08_04_sweco_bim_coordinator_antwerp</t>
+        </is>
+      </c>
+      <c r="R57" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S57" s="17" t="inlineStr">
+        <is>
+          <t>Strong direct BIM match. 3 years experience gap not disclosed per updated default; no language requirement listed.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="21">
       <c r="A58" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Sweco Sweden Information Coordinator row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5107,28 +5107,78 @@
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="21">
-      <c r="A58" s="11" t="n"/>
-      <c r="B58" s="11" t="n"/>
-      <c r="C58" s="11" t="n"/>
-      <c r="D58" s="12" t="n"/>
-      <c r="E58" s="11" t="n"/>
-      <c r="F58" s="11" t="n"/>
-      <c r="G58" s="11" t="n"/>
-      <c r="H58" s="13" t="n"/>
-      <c r="I58" s="12" t="n"/>
-      <c r="J58" s="12" t="n"/>
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>Sweco</t>
+        </is>
+      </c>
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>Information Coordinator (expression of interest)</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="inlineStr">
+        <is>
+          <t>Sundsvall/Ostersund, SE</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="inlineStr"/>
+      <c r="F58" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G58" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sweco.se/karriar/ansok-har/?rmpage=apply&amp;rmjob=25028</t>
+        </is>
+      </c>
+      <c r="H58" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I58" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J58" s="18" t="inlineStr"/>
       <c r="K58" s="14">
         <f>IF($H58="","",TODAY()-$H58)</f>
         <v/>
       </c>
-      <c r="L58" s="13" t="n"/>
-      <c r="M58" s="11" t="n"/>
-      <c r="N58" s="13" t="n"/>
-      <c r="O58" s="11" t="n"/>
-      <c r="P58" s="11" t="n"/>
-      <c r="Q58" s="11" t="n"/>
-      <c r="R58" s="12" t="n"/>
-      <c r="S58" s="11" t="n"/>
+      <c r="L58" s="19" t="inlineStr"/>
+      <c r="M58" s="17" t="inlineStr"/>
+      <c r="N58" s="19" t="inlineStr"/>
+      <c r="O58" s="17" t="inlineStr">
+        <is>
+          <t>Malin Kullstrom</t>
+        </is>
+      </c>
+      <c r="P58" s="17" t="inlineStr">
+        <is>
+          <t>malin.kullstrom@sweco.se</t>
+        </is>
+      </c>
+      <c r="Q58" s="17" t="inlineStr">
+        <is>
+          <t>sweden/2026_08_04_sweco_info_coordinator_sundsvall</t>
+        </is>
+      </c>
+      <c r="R58" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S58" s="17" t="inlineStr">
+        <is>
+          <t>Excellent domain fit — role is essentially the candidate’s exact specialty (Information Manager, ISO 19650). Swedish gap not disclosed per updated default; confirmed with user given the strong fit. 3 years experience also required.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="21">
       <c r="A59" s="11" t="n"/>

</xml_diff>

<commit_message>
Add WSP Junior Water Safety Advisor row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5181,28 +5181,66 @@
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="21">
-      <c r="A59" s="11" t="n"/>
-      <c r="B59" s="11" t="n"/>
-      <c r="C59" s="11" t="n"/>
-      <c r="D59" s="12" t="n"/>
-      <c r="E59" s="11" t="n"/>
-      <c r="F59" s="11" t="n"/>
-      <c r="G59" s="11" t="n"/>
-      <c r="H59" s="13" t="n"/>
-      <c r="I59" s="12" t="n"/>
-      <c r="J59" s="12" t="n"/>
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>WSP</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>Junior Water Safety Advisor – Water and Environment</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>Breda/Nieuwegein/Rotterdam, NL</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr"/>
+      <c r="F59" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G59" s="17" t="inlineStr"/>
+      <c r="H59" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I59" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J59" s="18" t="inlineStr"/>
       <c r="K59" s="14">
         <f>IF($H59="","",TODAY()-$H59)</f>
         <v/>
       </c>
-      <c r="L59" s="13" t="n"/>
-      <c r="M59" s="11" t="n"/>
-      <c r="N59" s="13" t="n"/>
-      <c r="O59" s="11" t="n"/>
-      <c r="P59" s="11" t="n"/>
-      <c r="Q59" s="11" t="n"/>
-      <c r="R59" s="12" t="n"/>
-      <c r="S59" s="11" t="n"/>
+      <c r="L59" s="19" t="inlineStr"/>
+      <c r="M59" s="17" t="inlineStr"/>
+      <c r="N59" s="19" t="inlineStr"/>
+      <c r="O59" s="17" t="inlineStr"/>
+      <c r="P59" s="17" t="inlineStr"/>
+      <c r="Q59" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_04_wsp_water_safety</t>
+        </is>
+      </c>
+      <c r="R59" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S59" s="17" t="inlineStr">
+        <is>
+          <t>First WSP application. Decent water-adjacent fit; geotechnical stability/piping analysis is a different specialty than hydrology coursework, framed honestly as genuine interest rather than claimed expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="21">
       <c r="A60" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Ferrovial BIM Graduate row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5243,28 +5243,70 @@
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="21">
-      <c r="A60" s="11" t="n"/>
-      <c r="B60" s="11" t="n"/>
-      <c r="C60" s="11" t="n"/>
-      <c r="D60" s="12" t="n"/>
-      <c r="E60" s="11" t="n"/>
-      <c r="F60" s="11" t="n"/>
-      <c r="G60" s="11" t="n"/>
-      <c r="H60" s="13" t="n"/>
-      <c r="I60" s="12" t="n"/>
-      <c r="J60" s="12" t="n"/>
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Ferrovial Construction</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>BIM Graduate – Quality and Design Department (JR18626)</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="inlineStr"/>
+      <c r="F60" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G60" s="17" t="inlineStr">
+        <is>
+          <t>https://ferrovial.wd3.myworkdayjobs.com/Ferrovial_Career_Site/job/London/BIM-Graduate_JR18626/apply?source=LinkedIn</t>
+        </is>
+      </c>
+      <c r="H60" s="19" t="n">
+        <v>46246</v>
+      </c>
+      <c r="I60" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J60" s="18" t="inlineStr"/>
       <c r="K60" s="14">
         <f>IF($H60="","",TODAY()-$H60)</f>
         <v/>
       </c>
-      <c r="L60" s="13" t="n"/>
-      <c r="M60" s="11" t="n"/>
-      <c r="N60" s="13" t="n"/>
-      <c r="O60" s="11" t="n"/>
-      <c r="P60" s="11" t="n"/>
-      <c r="Q60" s="11" t="n"/>
-      <c r="R60" s="12" t="n"/>
-      <c r="S60" s="11" t="n"/>
+      <c r="L60" s="19" t="inlineStr"/>
+      <c r="M60" s="17" t="inlineStr"/>
+      <c r="N60" s="19" t="inlineStr"/>
+      <c r="O60" s="17" t="inlineStr"/>
+      <c r="P60" s="17" t="inlineStr"/>
+      <c r="Q60" s="17" t="inlineStr">
+        <is>
+          <t>uk/2026_08_12_ferrovial_bim_graduate</t>
+        </is>
+      </c>
+      <c r="R60" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S60" s="17" t="inlineStr">
+        <is>
+          <t>Near-exact fit (posting names BIM as a qualifying master’s degree, 2-year graduate program, no experience required). UK right-to-work confirmed by user as securable by start date; stated directly on the CV per the posting’s essential requirement.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="21">
       <c r="A61" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Ferrovial Digital Construction & Data Management row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5309,28 +5309,70 @@
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="21">
-      <c r="A61" s="11" t="n"/>
-      <c r="B61" s="11" t="n"/>
-      <c r="C61" s="11" t="n"/>
-      <c r="D61" s="12" t="n"/>
-      <c r="E61" s="11" t="n"/>
-      <c r="F61" s="11" t="n"/>
-      <c r="G61" s="11" t="n"/>
-      <c r="H61" s="13" t="n"/>
-      <c r="I61" s="12" t="n"/>
-      <c r="J61" s="12" t="n"/>
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>Ferrovial Construction</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>Graduate Digital Construction &amp; Data Management 2026 (JR18262)</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="E61" s="17" t="inlineStr"/>
+      <c r="F61" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G61" s="17" t="inlineStr">
+        <is>
+          <t>https://ferrovial.wd3.myworkdayjobs.com/en-US/Ferrovial_Career_Site/job/London/Graduate-Digital-Construction---Data-Management-2026_JR18262/apply?source=LinkedIn</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="n">
+        <v>46246</v>
+      </c>
+      <c r="I61" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J61" s="18" t="inlineStr"/>
       <c r="K61" s="14">
         <f>IF($H61="","",TODAY()-$H61)</f>
         <v/>
       </c>
-      <c r="L61" s="13" t="n"/>
-      <c r="M61" s="11" t="n"/>
-      <c r="N61" s="13" t="n"/>
-      <c r="O61" s="11" t="n"/>
-      <c r="P61" s="11" t="n"/>
-      <c r="Q61" s="11" t="n"/>
-      <c r="R61" s="12" t="n"/>
-      <c r="S61" s="11" t="n"/>
+      <c r="L61" s="19" t="inlineStr"/>
+      <c r="M61" s="17" t="inlineStr"/>
+      <c r="N61" s="19" t="inlineStr"/>
+      <c r="O61" s="17" t="inlineStr"/>
+      <c r="P61" s="17" t="inlineStr"/>
+      <c r="Q61" s="17" t="inlineStr">
+        <is>
+          <t>uk/2026_08_12_ferrovial_digital_construction_data</t>
+        </is>
+      </c>
+      <c r="R61" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S61" s="17" t="inlineStr">
+        <is>
+          <t>Second Ferrovial application, same team/program as BIM Graduate (JR18626). UK right-to-work confirmed manageable by user, stated directly on CV.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="21">
       <c r="A62" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Graitec AEC Prototyping Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5375,28 +5375,62 @@
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="21">
-      <c r="A62" s="11" t="n"/>
-      <c r="B62" s="11" t="n"/>
-      <c r="C62" s="11" t="n"/>
-      <c r="D62" s="12" t="n"/>
-      <c r="E62" s="11" t="n"/>
-      <c r="F62" s="11" t="n"/>
-      <c r="G62" s="11" t="n"/>
-      <c r="H62" s="13" t="n"/>
-      <c r="I62" s="12" t="n"/>
-      <c r="J62" s="12" t="n"/>
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>Graitec</t>
+        </is>
+      </c>
+      <c r="B62" s="17" t="inlineStr">
+        <is>
+          <t>AEC Prototyping Engineer</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>Paris, FR</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr"/>
+      <c r="E62" s="17" t="inlineStr"/>
+      <c r="F62" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G62" s="17" t="inlineStr"/>
+      <c r="H62" s="19" t="n">
+        <v>46246</v>
+      </c>
+      <c r="I62" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J62" s="18" t="inlineStr"/>
       <c r="K62" s="14">
         <f>IF($H62="","",TODAY()-$H62)</f>
         <v/>
       </c>
-      <c r="L62" s="13" t="n"/>
-      <c r="M62" s="11" t="n"/>
-      <c r="N62" s="13" t="n"/>
-      <c r="O62" s="11" t="n"/>
-      <c r="P62" s="11" t="n"/>
-      <c r="Q62" s="11" t="n"/>
-      <c r="R62" s="12" t="n"/>
-      <c r="S62" s="11" t="n"/>
+      <c r="L62" s="19" t="inlineStr"/>
+      <c r="M62" s="17" t="inlineStr"/>
+      <c r="N62" s="19" t="inlineStr"/>
+      <c r="O62" s="17" t="inlineStr"/>
+      <c r="P62" s="17" t="inlineStr"/>
+      <c r="Q62" s="17" t="inlineStr">
+        <is>
+          <t>france/2026_08_12_graitec_aec_prototyping</t>
+        </is>
+      </c>
+      <c r="R62" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S62" s="17" t="inlineStr">
+        <is>
+          <t>Exceptional fit — combines both core specialties (AEC/BIM and AI/agentic systems). BIMGraphExplorer is an almost literal match to the role’s rapid-prototyping/validation cycle. No French requirement listed.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="21">
       <c r="A63" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Mott MacDonald BIM Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5433,28 +5433,74 @@
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="21">
-      <c r="A63" s="11" t="n"/>
-      <c r="B63" s="11" t="n"/>
-      <c r="C63" s="11" t="n"/>
-      <c r="D63" s="12" t="n"/>
-      <c r="E63" s="11" t="n"/>
-      <c r="F63" s="11" t="n"/>
-      <c r="G63" s="11" t="n"/>
-      <c r="H63" s="13" t="n"/>
-      <c r="I63" s="12" t="n"/>
-      <c r="J63" s="12" t="n"/>
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>Mott MacDonald</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>BIM Engineer (Structural BIM), Energy unit (Job Ref 15395)</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>Sofia, BG</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr"/>
+      <c r="F63" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>https://career2.successfactors.eu/career?company=MMPROD&amp;lang=en_150&amp;login_ns=register&amp;career_ns=job_application&amp;career_job_req_id=15395&amp;jobPipeline=CareerSite&amp;codes=EXT</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I63" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J63" s="18" t="inlineStr"/>
       <c r="K63" s="14">
         <f>IF($H63="","",TODAY()-$H63)</f>
         <v/>
       </c>
-      <c r="L63" s="13" t="n"/>
-      <c r="M63" s="11" t="n"/>
-      <c r="N63" s="13" t="n"/>
-      <c r="O63" s="11" t="n"/>
-      <c r="P63" s="11" t="n"/>
-      <c r="Q63" s="11" t="n"/>
-      <c r="R63" s="12" t="n"/>
-      <c r="S63" s="11" t="n"/>
+      <c r="L63" s="19" t="inlineStr"/>
+      <c r="M63" s="17" t="inlineStr"/>
+      <c r="N63" s="19" t="inlineStr"/>
+      <c r="O63" s="17" t="inlineStr">
+        <is>
+          <t>Maria Cervantes</t>
+        </is>
+      </c>
+      <c r="P63" s="17" t="inlineStr"/>
+      <c r="Q63" s="17" t="inlineStr">
+        <is>
+          <t>bulgaria/2026_08_16_mott_macdonald_bim_sofia</t>
+        </is>
+      </c>
+      <c r="R63" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S63" s="17" t="inlineStr">
+        <is>
+          <t>Structural-engineering degree gap not disclosed per updated default; actual day-to-day tasks (ACC, ISO 19650, clash detection) map very well to real strengths.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="21">
       <c r="A64" s="11" t="n"/>

</xml_diff>

<commit_message>
Add AECOM BIM & Digital Specialist row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5503,28 +5503,66 @@
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="21">
-      <c r="A64" s="11" t="n"/>
-      <c r="B64" s="11" t="n"/>
-      <c r="C64" s="11" t="n"/>
-      <c r="D64" s="12" t="n"/>
-      <c r="E64" s="11" t="n"/>
-      <c r="F64" s="11" t="n"/>
-      <c r="G64" s="11" t="n"/>
-      <c r="H64" s="13" t="n"/>
-      <c r="I64" s="12" t="n"/>
-      <c r="J64" s="12" t="n"/>
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>AECOM</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>BIM &amp; Digital Specialist / Digital Project Delivery Engineer (Req J10154523)</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="inlineStr">
+        <is>
+          <t>Madrid, ES</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="inlineStr"/>
+      <c r="F64" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G64" s="17" t="inlineStr"/>
+      <c r="H64" s="19" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I64" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J64" s="18" t="inlineStr"/>
       <c r="K64" s="14">
         <f>IF($H64="","",TODAY()-$H64)</f>
         <v/>
       </c>
-      <c r="L64" s="13" t="n"/>
-      <c r="M64" s="11" t="n"/>
-      <c r="N64" s="13" t="n"/>
-      <c r="O64" s="11" t="n"/>
-      <c r="P64" s="11" t="n"/>
-      <c r="Q64" s="11" t="n"/>
-      <c r="R64" s="12" t="n"/>
-      <c r="S64" s="11" t="n"/>
+      <c r="L64" s="19" t="inlineStr"/>
+      <c r="M64" s="17" t="inlineStr"/>
+      <c r="N64" s="19" t="inlineStr"/>
+      <c r="O64" s="17" t="inlineStr"/>
+      <c r="P64" s="17" t="inlineStr"/>
+      <c r="Q64" s="17" t="inlineStr">
+        <is>
+          <t>spain/2026_08_16_aecom_bim_digital_madrid</t>
+        </is>
+      </c>
+      <c r="R64" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S64" s="17" t="inlineStr">
+        <is>
+          <t>Good BIM+data/automation fit (similar shape to Graitec). 2-5 years experience and Power Platform/Azure gaps not disclosed per updated default; no Spanish requirement stated, only English.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="21">
       <c r="A65" s="11" t="n"/>

</xml_diff>

<commit_message>
Add King and Moffatt Engineering Graduate Programme row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5565,28 +5565,66 @@
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="21">
-      <c r="A65" s="11" t="n"/>
-      <c r="B65" s="11" t="n"/>
-      <c r="C65" s="11" t="n"/>
-      <c r="D65" s="12" t="n"/>
-      <c r="E65" s="11" t="n"/>
-      <c r="F65" s="11" t="n"/>
-      <c r="G65" s="11" t="n"/>
-      <c r="H65" s="13" t="n"/>
-      <c r="I65" s="12" t="n"/>
-      <c r="J65" s="12" t="n"/>
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>King and Moffatt Building Services</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>Engineering Graduate Programme</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="inlineStr">
+        <is>
+          <t>Carrick-on-Shannon, Co. Leitrim, IE</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr"/>
+      <c r="F65" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G65" s="17" t="inlineStr"/>
+      <c r="H65" s="19" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I65" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J65" s="18" t="inlineStr"/>
       <c r="K65" s="14">
         <f>IF($H65="","",TODAY()-$H65)</f>
         <v/>
       </c>
-      <c r="L65" s="13" t="n"/>
-      <c r="M65" s="11" t="n"/>
-      <c r="N65" s="13" t="n"/>
-      <c r="O65" s="11" t="n"/>
-      <c r="P65" s="11" t="n"/>
-      <c r="Q65" s="11" t="n"/>
-      <c r="R65" s="12" t="n"/>
-      <c r="S65" s="11" t="n"/>
+      <c r="L65" s="19" t="inlineStr"/>
+      <c r="M65" s="17" t="inlineStr"/>
+      <c r="N65" s="19" t="inlineStr"/>
+      <c r="O65" s="17" t="inlineStr"/>
+      <c r="P65" s="17" t="inlineStr"/>
+      <c r="Q65" s="17" t="inlineStr">
+        <is>
+          <t>ireland/2026_08_16_king_moffatt_engineering_graduate</t>
+        </is>
+      </c>
+      <c r="R65" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S65" s="17" t="inlineStr">
+        <is>
+          <t>Ireland work-authorization status unresolved — user asked to omit any mention either way, to be sorted out separately. Also a degree-field mismatch (M&amp;E/Building Services vs Civil), bridged via the programme’s Design/BIM rotation.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="21">
       <c r="A66" s="11" t="n"/>

</xml_diff>

<commit_message>
Add DBFL Graduate Development Programme row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5627,28 +5627,62 @@
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="21">
-      <c r="A66" s="11" t="n"/>
-      <c r="B66" s="11" t="n"/>
-      <c r="C66" s="11" t="n"/>
-      <c r="D66" s="12" t="n"/>
-      <c r="E66" s="11" t="n"/>
-      <c r="F66" s="11" t="n"/>
-      <c r="G66" s="11" t="n"/>
-      <c r="H66" s="13" t="n"/>
-      <c r="I66" s="12" t="n"/>
-      <c r="J66" s="12" t="n"/>
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>DBFL Consulting Engineers</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>Graduate Development Programme</t>
+        </is>
+      </c>
+      <c r="C66" s="17" t="inlineStr">
+        <is>
+          <t>Dublin, IE</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr"/>
+      <c r="E66" s="17" t="inlineStr"/>
+      <c r="F66" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G66" s="17" t="inlineStr"/>
+      <c r="H66" s="19" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I66" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J66" s="18" t="inlineStr"/>
       <c r="K66" s="14">
         <f>IF($H66="","",TODAY()-$H66)</f>
         <v/>
       </c>
-      <c r="L66" s="13" t="n"/>
-      <c r="M66" s="11" t="n"/>
-      <c r="N66" s="13" t="n"/>
-      <c r="O66" s="11" t="n"/>
-      <c r="P66" s="11" t="n"/>
-      <c r="Q66" s="11" t="n"/>
-      <c r="R66" s="12" t="n"/>
-      <c r="S66" s="11" t="n"/>
+      <c r="L66" s="19" t="inlineStr"/>
+      <c r="M66" s="17" t="inlineStr"/>
+      <c r="N66" s="19" t="inlineStr"/>
+      <c r="O66" s="17" t="inlineStr"/>
+      <c r="P66" s="17" t="inlineStr"/>
+      <c r="Q66" s="17" t="inlineStr">
+        <is>
+          <t>ireland/2026_08_16_dbfl_graduate_programme</t>
+        </is>
+      </c>
+      <c r="R66" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S66" s="17" t="inlineStr">
+        <is>
+          <t>Strong degree-field match (pure Civil Engineering). Same unresolved Ireland work-authorization question as King and Moffatt; omitted from CV per user instruction.</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="21">
       <c r="A67" s="11" t="n"/>

</xml_diff>

<commit_message>
Add TwinMaster Product Manager row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5685,28 +5685,74 @@
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="21">
-      <c r="A67" s="11" t="n"/>
-      <c r="B67" s="11" t="n"/>
-      <c r="C67" s="11" t="n"/>
-      <c r="D67" s="12" t="n"/>
-      <c r="E67" s="11" t="n"/>
-      <c r="F67" s="11" t="n"/>
-      <c r="G67" s="11" t="n"/>
-      <c r="H67" s="13" t="n"/>
-      <c r="I67" s="12" t="n"/>
-      <c r="J67" s="12" t="n"/>
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>TwinMaster</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>Product Manager (Arch-e platform)</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E67" s="17" t="inlineStr"/>
+      <c r="F67" s="17" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G67" s="17" t="inlineStr"/>
+      <c r="H67" s="19" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I67" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J67" s="18" t="inlineStr"/>
       <c r="K67" s="14">
         <f>IF($H67="","",TODAY()-$H67)</f>
         <v/>
       </c>
-      <c r="L67" s="13" t="n"/>
-      <c r="M67" s="11" t="n"/>
-      <c r="N67" s="13" t="n"/>
-      <c r="O67" s="11" t="n"/>
-      <c r="P67" s="11" t="n"/>
-      <c r="Q67" s="11" t="n"/>
-      <c r="R67" s="12" t="n"/>
-      <c r="S67" s="11" t="n"/>
+      <c r="L67" s="19" t="inlineStr"/>
+      <c r="M67" s="17" t="inlineStr"/>
+      <c r="N67" s="19" t="inlineStr"/>
+      <c r="O67" s="17" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="P67" s="17" t="inlineStr">
+        <is>
+          <t>michael@thetwinmaster.com</t>
+        </is>
+      </c>
+      <c r="Q67" s="17" t="inlineStr">
+        <is>
+          <t>remote/2026_08_16_twinmaster_product_manager</t>
+        </is>
+      </c>
+      <c r="R67" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S67" s="17" t="inlineStr">
+        <is>
+          <t>Categorical mismatch (Licensed Architect, 7 years, Architect of Record required). Sent as an openly self-aware networking note rather than a standard tailored pitch, per explicit user direction.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="21">
       <c r="A68" s="11" t="n"/>

</xml_diff>

<commit_message>
Add BAM BIM Coordinator row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5755,28 +5755,62 @@
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="21">
-      <c r="A68" s="11" t="n"/>
-      <c r="B68" s="11" t="n"/>
-      <c r="C68" s="11" t="n"/>
-      <c r="D68" s="12" t="n"/>
-      <c r="E68" s="11" t="n"/>
-      <c r="F68" s="11" t="n"/>
-      <c r="G68" s="11" t="n"/>
-      <c r="H68" s="13" t="n"/>
-      <c r="I68" s="12" t="n"/>
-      <c r="J68" s="12" t="n"/>
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>BAM Building</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="inlineStr">
+        <is>
+          <t>BIM Coordinator (Digital Project Solutions)</t>
+        </is>
+      </c>
+      <c r="C68" s="17" t="inlineStr">
+        <is>
+          <t>Waterford, IE</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr"/>
+      <c r="E68" s="17" t="inlineStr"/>
+      <c r="F68" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G68" s="17" t="inlineStr"/>
+      <c r="H68" s="19" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I68" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J68" s="18" t="inlineStr"/>
       <c r="K68" s="14">
         <f>IF($H68="","",TODAY()-$H68)</f>
         <v/>
       </c>
-      <c r="L68" s="13" t="n"/>
-      <c r="M68" s="11" t="n"/>
-      <c r="N68" s="13" t="n"/>
-      <c r="O68" s="11" t="n"/>
-      <c r="P68" s="11" t="n"/>
-      <c r="Q68" s="11" t="n"/>
-      <c r="R68" s="12" t="n"/>
-      <c r="S68" s="11" t="n"/>
+      <c r="L68" s="19" t="inlineStr"/>
+      <c r="M68" s="17" t="inlineStr"/>
+      <c r="N68" s="19" t="inlineStr"/>
+      <c r="O68" s="17" t="inlineStr"/>
+      <c r="P68" s="17" t="inlineStr"/>
+      <c r="Q68" s="17" t="inlineStr">
+        <is>
+          <t>ireland/2026_08_16_bam_bim_coordinator_waterford</t>
+        </is>
+      </c>
+      <c r="R68" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S68" s="17" t="inlineStr">
+        <is>
+          <t>Excellent direct match — ISO 19650/CDE/MIDP-TIDP is the candidate’s core specialty. Same unresolved Ireland work-authorization question as King and Moffatt/DBFL; omitted from CV per user instruction.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="21">
       <c r="A69" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Hurks/Ballast Nedam BIM Coordinator row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5813,28 +5813,74 @@
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="21">
-      <c r="A69" s="11" t="n"/>
-      <c r="B69" s="11" t="n"/>
-      <c r="C69" s="11" t="n"/>
-      <c r="D69" s="12" t="n"/>
-      <c r="E69" s="11" t="n"/>
-      <c r="F69" s="11" t="n"/>
-      <c r="G69" s="11" t="n"/>
-      <c r="H69" s="13" t="n"/>
-      <c r="I69" s="12" t="n"/>
-      <c r="J69" s="12" t="n"/>
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>Hurks (Ballast Nedam)</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>BIM Coordinator</t>
+        </is>
+      </c>
+      <c r="C69" s="17" t="inlineStr">
+        <is>
+          <t>Eindhoven, NL</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr">
+        <is>
+          <t>EUR 3,989-5,699/month</t>
+        </is>
+      </c>
+      <c r="F69" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G69" s="17" t="inlineStr"/>
+      <c r="H69" s="19" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I69" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J69" s="18" t="inlineStr"/>
       <c r="K69" s="14">
         <f>IF($H69="","",TODAY()-$H69)</f>
         <v/>
       </c>
-      <c r="L69" s="13" t="n"/>
-      <c r="M69" s="11" t="n"/>
-      <c r="N69" s="13" t="n"/>
-      <c r="O69" s="11" t="n"/>
-      <c r="P69" s="11" t="n"/>
-      <c r="Q69" s="11" t="n"/>
-      <c r="R69" s="12" t="n"/>
-      <c r="S69" s="11" t="n"/>
+      <c r="L69" s="19" t="inlineStr"/>
+      <c r="M69" s="17" t="inlineStr"/>
+      <c r="N69" s="19" t="inlineStr"/>
+      <c r="O69" s="17" t="inlineStr">
+        <is>
+          <t>Anneke den Haan</t>
+        </is>
+      </c>
+      <c r="P69" s="17" t="inlineStr"/>
+      <c r="Q69" s="17" t="inlineStr">
+        <is>
+          <t>netherlands/2026_08_16_hurks_ballast_nedam_bim</t>
+        </is>
+      </c>
+      <c r="R69" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S69" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn flagged this as a "low" match (missing years of experience, specific tools: Solibri/BIMcollab Nexus/Dalux, Dutch fluency). Not disclosed per updated default; leans on genuine BIM/ISO19650/AI overlap.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="21">
       <c r="A70" s="11" t="n"/>

</xml_diff>

<commit_message>
Add REM d.o.o. Designer-Developer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5883,28 +5883,62 @@
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="21">
-      <c r="A70" s="11" t="n"/>
-      <c r="B70" s="11" t="n"/>
-      <c r="C70" s="11" t="n"/>
-      <c r="D70" s="12" t="n"/>
-      <c r="E70" s="11" t="n"/>
-      <c r="F70" s="11" t="n"/>
-      <c r="G70" s="11" t="n"/>
-      <c r="H70" s="13" t="n"/>
-      <c r="I70" s="12" t="n"/>
-      <c r="J70" s="12" t="n"/>
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>REM d.o.o.</t>
+        </is>
+      </c>
+      <c r="B70" s="17" t="inlineStr">
+        <is>
+          <t>Designer-Developer (product design/development)</t>
+        </is>
+      </c>
+      <c r="C70" s="17" t="inlineStr">
+        <is>
+          <t>Trebnje, SI</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr"/>
+      <c r="E70" s="17" t="inlineStr"/>
+      <c r="F70" s="17" t="inlineStr">
+        <is>
+          <t>Job Board</t>
+        </is>
+      </c>
+      <c r="G70" s="17" t="inlineStr"/>
+      <c r="H70" s="19" t="n">
+        <v>46251</v>
+      </c>
+      <c r="I70" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J70" s="18" t="inlineStr"/>
       <c r="K70" s="14">
         <f>IF($H70="","",TODAY()-$H70)</f>
         <v/>
       </c>
-      <c r="L70" s="13" t="n"/>
-      <c r="M70" s="11" t="n"/>
-      <c r="N70" s="13" t="n"/>
-      <c r="O70" s="11" t="n"/>
-      <c r="P70" s="11" t="n"/>
-      <c r="Q70" s="11" t="n"/>
-      <c r="R70" s="12" t="n"/>
-      <c r="S70" s="11" t="n"/>
+      <c r="L70" s="19" t="inlineStr"/>
+      <c r="M70" s="17" t="inlineStr"/>
+      <c r="N70" s="19" t="inlineStr"/>
+      <c r="O70" s="17" t="inlineStr"/>
+      <c r="P70" s="17" t="inlineStr"/>
+      <c r="Q70" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_08_17_rem_doo_trebnje</t>
+        </is>
+      </c>
+      <c r="R70" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S70" s="17" t="inlineStr">
+        <is>
+          <t>Good fit for modular building systems manufacturer. Revit explicitly named; English satisfies language requirement (no Slovene needed). 2 years experience gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="21">
       <c r="A71" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Pilon AEC open application row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -5941,28 +5941,70 @@
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="21">
-      <c r="A71" s="11" t="n"/>
-      <c r="B71" s="11" t="n"/>
-      <c r="C71" s="11" t="n"/>
-      <c r="D71" s="12" t="n"/>
-      <c r="E71" s="11" t="n"/>
-      <c r="F71" s="11" t="n"/>
-      <c r="G71" s="11" t="n"/>
-      <c r="H71" s="13" t="n"/>
-      <c r="I71" s="12" t="n"/>
-      <c r="J71" s="12" t="n"/>
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>Pilon AEC</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="inlineStr">
+        <is>
+          <t>Open application – BIM specialist</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>Ljubljana, SI</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr"/>
+      <c r="E71" s="17" t="inlineStr"/>
+      <c r="F71" s="17" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G71" s="17" t="inlineStr">
+        <is>
+          <t>https://www.pilon.si/</t>
+        </is>
+      </c>
+      <c r="H71" s="19" t="n">
+        <v>46251</v>
+      </c>
+      <c r="I71" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J71" s="18" t="inlineStr"/>
       <c r="K71" s="14">
         <f>IF($H71="","",TODAY()-$H71)</f>
         <v/>
       </c>
-      <c r="L71" s="13" t="n"/>
-      <c r="M71" s="11" t="n"/>
-      <c r="N71" s="13" t="n"/>
-      <c r="O71" s="11" t="n"/>
-      <c r="P71" s="11" t="n"/>
-      <c r="Q71" s="11" t="n"/>
-      <c r="R71" s="12" t="n"/>
-      <c r="S71" s="11" t="n"/>
+      <c r="L71" s="19" t="inlineStr"/>
+      <c r="M71" s="17" t="inlineStr"/>
+      <c r="N71" s="19" t="inlineStr"/>
+      <c r="O71" s="17" t="inlineStr"/>
+      <c r="P71" s="17" t="inlineStr">
+        <is>
+          <t>info@pilon.si</t>
+        </is>
+      </c>
+      <c r="Q71" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_08_17_pilon_open_application</t>
+        </is>
+      </c>
+      <c r="R71" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S71" s="17" t="inlineStr">
+        <is>
+          <t>Genuine speculative pitch to a real BIM software company (Archicad/MEP Designer/DDScad distributor). Stronger fit than Atrij/Saning since Pilon’s core business is BIM. No named contact or careers page found.</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="21">
       <c r="A72" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Geoservis open application row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6007,28 +6007,70 @@
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="21">
-      <c r="A72" s="11" t="n"/>
-      <c r="B72" s="11" t="n"/>
-      <c r="C72" s="11" t="n"/>
-      <c r="D72" s="12" t="n"/>
-      <c r="E72" s="11" t="n"/>
-      <c r="F72" s="11" t="n"/>
-      <c r="G72" s="11" t="n"/>
-      <c r="H72" s="13" t="n"/>
-      <c r="I72" s="12" t="n"/>
-      <c r="J72" s="12" t="n"/>
+      <c r="A72" s="17" t="inlineStr">
+        <is>
+          <t>Geoservis d.o.o.</t>
+        </is>
+      </c>
+      <c r="B72" s="17" t="inlineStr">
+        <is>
+          <t>Open application – BIM and geospatial background</t>
+        </is>
+      </c>
+      <c r="C72" s="17" t="inlineStr">
+        <is>
+          <t>Ljubljana, SI</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr"/>
+      <c r="E72" s="17" t="inlineStr"/>
+      <c r="F72" s="17" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G72" s="17" t="inlineStr">
+        <is>
+          <t>https://geoservis.si/</t>
+        </is>
+      </c>
+      <c r="H72" s="19" t="n">
+        <v>46251</v>
+      </c>
+      <c r="I72" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J72" s="18" t="inlineStr"/>
       <c r="K72" s="14">
         <f>IF($H72="","",TODAY()-$H72)</f>
         <v/>
       </c>
-      <c r="L72" s="13" t="n"/>
-      <c r="M72" s="11" t="n"/>
-      <c r="N72" s="13" t="n"/>
-      <c r="O72" s="11" t="n"/>
-      <c r="P72" s="11" t="n"/>
-      <c r="Q72" s="11" t="n"/>
-      <c r="R72" s="12" t="n"/>
-      <c r="S72" s="11" t="n"/>
+      <c r="L72" s="19" t="inlineStr"/>
+      <c r="M72" s="17" t="inlineStr"/>
+      <c r="N72" s="19" t="inlineStr"/>
+      <c r="O72" s="17" t="inlineStr"/>
+      <c r="P72" s="17" t="inlineStr">
+        <is>
+          <t>info@geoservis.si</t>
+        </is>
+      </c>
+      <c r="Q72" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_08_17_geoservis_open_application</t>
+        </is>
+      </c>
+      <c r="R72" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S72" s="17" t="inlineStr">
+        <is>
+          <t>Speculative pitch to a Leica Geosystems surveying/3D-scanning equipment distributor. Genuine fit via real scan-to-BIM point-cloud coursework and ArcGIS. No named contact or careers page found.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="21">
       <c r="A73" s="11" t="n"/>

</xml_diff>

<commit_message>
Add BIMING open application row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6073,28 +6073,74 @@
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="21">
-      <c r="A73" s="11" t="n"/>
-      <c r="B73" s="11" t="n"/>
-      <c r="C73" s="11" t="n"/>
-      <c r="D73" s="12" t="n"/>
-      <c r="E73" s="11" t="n"/>
-      <c r="F73" s="11" t="n"/>
-      <c r="G73" s="11" t="n"/>
-      <c r="H73" s="13" t="n"/>
-      <c r="I73" s="12" t="n"/>
-      <c r="J73" s="12" t="n"/>
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>BIMING (Epoha d.o.o.)</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="inlineStr">
+        <is>
+          <t>Open application – scan-to-BIM background</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>Ljubljana, SI</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr"/>
+      <c r="E73" s="17" t="inlineStr"/>
+      <c r="F73" s="17" t="inlineStr">
+        <is>
+          <t>Networking</t>
+        </is>
+      </c>
+      <c r="G73" s="17" t="inlineStr">
+        <is>
+          <t>https://biming.si/</t>
+        </is>
+      </c>
+      <c r="H73" s="19" t="n">
+        <v>46251</v>
+      </c>
+      <c r="I73" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J73" s="18" t="inlineStr"/>
       <c r="K73" s="14">
         <f>IF($H73="","",TODAY()-$H73)</f>
         <v/>
       </c>
-      <c r="L73" s="13" t="n"/>
-      <c r="M73" s="11" t="n"/>
-      <c r="N73" s="13" t="n"/>
-      <c r="O73" s="11" t="n"/>
-      <c r="P73" s="11" t="n"/>
-      <c r="Q73" s="11" t="n"/>
-      <c r="R73" s="12" t="n"/>
-      <c r="S73" s="11" t="n"/>
+      <c r="L73" s="19" t="inlineStr"/>
+      <c r="M73" s="17" t="inlineStr"/>
+      <c r="N73" s="19" t="inlineStr"/>
+      <c r="O73" s="17" t="inlineStr">
+        <is>
+          <t>Gregor Novakovic</t>
+        </is>
+      </c>
+      <c r="P73" s="17" t="inlineStr">
+        <is>
+          <t>info@epoha.si</t>
+        </is>
+      </c>
+      <c r="Q73" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_08_17_biming_gregor_novakovic</t>
+        </is>
+      </c>
+      <c r="R73" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S73" s="17" t="inlineStr">
+        <is>
+          <t>Exceptional fit — BIMING’s core business (point-cloud to BIM conversion) almost literally matches the candidate’s scan-to-BIM coursework. Addressed to named CEO.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="21">
       <c r="A74" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Hilti Technical Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6143,28 +6143,66 @@
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="21">
-      <c r="A74" s="11" t="n"/>
-      <c r="B74" s="11" t="n"/>
-      <c r="C74" s="11" t="n"/>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="11" t="n"/>
-      <c r="F74" s="11" t="n"/>
-      <c r="G74" s="11" t="n"/>
-      <c r="H74" s="13" t="n"/>
-      <c r="I74" s="12" t="n"/>
-      <c r="J74" s="12" t="n"/>
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>Hilti</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>Technical Engineer (Req. 18545)</t>
+        </is>
+      </c>
+      <c r="C74" s="17" t="inlineStr">
+        <is>
+          <t>Trzin, SI</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr"/>
+      <c r="E74" s="17" t="inlineStr"/>
+      <c r="F74" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G74" s="17" t="inlineStr">
+        <is>
+          <t>https://careers.hilti.group/en/jobs/</t>
+        </is>
+      </c>
+      <c r="H74" s="19" t="n">
+        <v>46251</v>
+      </c>
+      <c r="I74" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J74" s="18" t="inlineStr"/>
       <c r="K74" s="14">
         <f>IF($H74="","",TODAY()-$H74)</f>
         <v/>
       </c>
-      <c r="L74" s="13" t="n"/>
-      <c r="M74" s="11" t="n"/>
-      <c r="N74" s="13" t="n"/>
-      <c r="O74" s="11" t="n"/>
-      <c r="P74" s="11" t="n"/>
-      <c r="Q74" s="11" t="n"/>
-      <c r="R74" s="12" t="n"/>
-      <c r="S74" s="11" t="n"/>
+      <c r="L74" s="19" t="inlineStr"/>
+      <c r="M74" s="17" t="inlineStr"/>
+      <c r="N74" s="19" t="inlineStr"/>
+      <c r="O74" s="17" t="inlineStr"/>
+      <c r="P74" s="17" t="inlineStr"/>
+      <c r="Q74" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_08_17_hilti_technical_engineer</t>
+        </is>
+      </c>
+      <c r="R74" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S74" s="17" t="inlineStr">
+        <is>
+          <t>General civil-engineering technical-consulting fit, not BIM-specific. Driving license omitted per standing instruction; 2 years experience gap not disclosed per updated default.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="21">
       <c r="A75" s="11" t="n"/>

</xml_diff>

<commit_message>
Add ELES CDE Administrator row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6205,28 +6205,66 @@
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="21">
-      <c r="A75" s="11" t="n"/>
-      <c r="B75" s="11" t="n"/>
-      <c r="C75" s="11" t="n"/>
-      <c r="D75" s="12" t="n"/>
-      <c r="E75" s="11" t="n"/>
-      <c r="F75" s="11" t="n"/>
-      <c r="G75" s="11" t="n"/>
-      <c r="H75" s="13" t="n"/>
-      <c r="I75" s="12" t="n"/>
-      <c r="J75" s="12" t="n"/>
+      <c r="A75" s="17" t="inlineStr">
+        <is>
+          <t>ELES, d.o.o.</t>
+        </is>
+      </c>
+      <c r="B75" s="17" t="inlineStr">
+        <is>
+          <t>Administrator skupnega podatkovnega okolja (CDE/Dalux Administrator) — student work</t>
+        </is>
+      </c>
+      <c r="C75" s="17" t="inlineStr">
+        <is>
+          <t>Ljubljana (Bericevo), SI</t>
+        </is>
+      </c>
+      <c r="D75" s="18" t="n"/>
+      <c r="E75" s="17" t="n"/>
+      <c r="F75" s="17" t="inlineStr">
+        <is>
+          <t>Job Board</t>
+        </is>
+      </c>
+      <c r="G75" s="17" t="inlineStr">
+        <is>
+          <t>https://www.eles.si/</t>
+        </is>
+      </c>
+      <c r="H75" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="I75" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J75" s="18" t="n"/>
       <c r="K75" s="14">
         <f>IF($H75="","",TODAY()-$H75)</f>
         <v/>
       </c>
-      <c r="L75" s="13" t="n"/>
-      <c r="M75" s="11" t="n"/>
-      <c r="N75" s="13" t="n"/>
-      <c r="O75" s="11" t="n"/>
-      <c r="P75" s="11" t="n"/>
-      <c r="Q75" s="11" t="n"/>
-      <c r="R75" s="12" t="n"/>
-      <c r="S75" s="11" t="n"/>
+      <c r="L75" s="19" t="n"/>
+      <c r="M75" s="17" t="n"/>
+      <c r="N75" s="19" t="n"/>
+      <c r="O75" s="17" t="n"/>
+      <c r="P75" s="17" t="n"/>
+      <c r="Q75" s="17" t="inlineStr">
+        <is>
+          <t>slovenia/2026_08_19_eles_cde_administrator</t>
+        </is>
+      </c>
+      <c r="R75" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S75" s="17" t="inlineStr">
+        <is>
+          <t>Strong fit: student role administering the CDE (Dalux) for an active BIM implementation project, explicitly targeting BIM-trained master's students. Profile led with CDE administration and ISO 19650 EIR validation experience.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="21">
       <c r="A76" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Winthrop Technologies BIM Technician row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6267,28 +6267,66 @@
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="21">
-      <c r="A76" s="11" t="n"/>
-      <c r="B76" s="11" t="n"/>
-      <c r="C76" s="11" t="n"/>
-      <c r="D76" s="12" t="n"/>
-      <c r="E76" s="11" t="n"/>
-      <c r="F76" s="11" t="n"/>
-      <c r="G76" s="11" t="n"/>
-      <c r="H76" s="13" t="n"/>
-      <c r="I76" s="12" t="n"/>
-      <c r="J76" s="12" t="n"/>
+      <c r="A76" s="17" t="inlineStr">
+        <is>
+          <t>Winthrop Technologies</t>
+        </is>
+      </c>
+      <c r="B76" s="17" t="inlineStr">
+        <is>
+          <t>BIM Technician (MEP bias)</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="inlineStr">
+        <is>
+          <t>Ballymount, Dublin 22, IE</t>
+        </is>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>Office-based (5 days/week)</t>
+        </is>
+      </c>
+      <c r="E76" s="17" t="n"/>
+      <c r="F76" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G76" s="17" t="n"/>
+      <c r="H76" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="I76" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J76" s="18" t="n"/>
       <c r="K76" s="14">
         <f>IF($H76="","",TODAY()-$H76)</f>
         <v/>
       </c>
-      <c r="L76" s="13" t="n"/>
-      <c r="M76" s="11" t="n"/>
-      <c r="N76" s="13" t="n"/>
-      <c r="O76" s="11" t="n"/>
-      <c r="P76" s="11" t="n"/>
-      <c r="Q76" s="11" t="n"/>
-      <c r="R76" s="12" t="n"/>
-      <c r="S76" s="11" t="n"/>
+      <c r="L76" s="19" t="n"/>
+      <c r="M76" s="17" t="n"/>
+      <c r="N76" s="19" t="n"/>
+      <c r="O76" s="17" t="n"/>
+      <c r="P76" s="17" t="n"/>
+      <c r="Q76" s="17" t="inlineStr">
+        <is>
+          <t>ireland/2026_08_19_winthrop_bim_technician</t>
+        </is>
+      </c>
+      <c r="R76" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S76" s="17" t="inlineStr">
+        <is>
+          <t>Genuine tools fit (Revit, AutoCAD, MEP clash detection, ISO 19650 EIR), but posting asks for 2 years' MEP BIM experience and Navisworks, which are gaps not disclosed per standing policy.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="21">
       <c r="A77" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Winthrop Graduate CSA Engineer row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6329,28 +6329,62 @@
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="21">
-      <c r="A77" s="11" t="n"/>
-      <c r="B77" s="11" t="n"/>
-      <c r="C77" s="11" t="n"/>
-      <c r="D77" s="12" t="n"/>
-      <c r="E77" s="11" t="n"/>
-      <c r="F77" s="11" t="n"/>
-      <c r="G77" s="11" t="n"/>
-      <c r="H77" s="13" t="n"/>
-      <c r="I77" s="12" t="n"/>
-      <c r="J77" s="12" t="n"/>
+      <c r="A77" s="17" t="inlineStr">
+        <is>
+          <t>Winthrop Technologies</t>
+        </is>
+      </c>
+      <c r="B77" s="17" t="inlineStr">
+        <is>
+          <t>Graduate CSA Engineer 2026</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="inlineStr">
+        <is>
+          <t>Dublin, IE</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="n"/>
+      <c r="E77" s="17" t="n"/>
+      <c r="F77" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G77" s="17" t="n"/>
+      <c r="H77" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="I77" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J77" s="18" t="n"/>
       <c r="K77" s="14">
         <f>IF($H77="","",TODAY()-$H77)</f>
         <v/>
       </c>
-      <c r="L77" s="13" t="n"/>
-      <c r="M77" s="11" t="n"/>
-      <c r="N77" s="13" t="n"/>
-      <c r="O77" s="11" t="n"/>
-      <c r="P77" s="11" t="n"/>
-      <c r="Q77" s="11" t="n"/>
-      <c r="R77" s="12" t="n"/>
-      <c r="S77" s="11" t="n"/>
+      <c r="L77" s="19" t="n"/>
+      <c r="M77" s="17" t="n"/>
+      <c r="N77" s="19" t="n"/>
+      <c r="O77" s="17" t="n"/>
+      <c r="P77" s="17" t="n"/>
+      <c r="Q77" s="17" t="inlineStr">
+        <is>
+          <t>ireland/2026_08_19_winthrop_graduate_csa</t>
+        </is>
+      </c>
+      <c r="R77" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S77" s="17" t="inlineStr">
+        <is>
+          <t>Strong graduate-programme fit: civil engineering degree plus drawing-review and design-coordination experience map directly onto CSA responsibilities. Second application to Winthrop (also applied to BIM Technician role).</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="21">
       <c r="A78" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Poperinge Junior Project Leader row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6387,28 +6387,62 @@
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="21">
-      <c r="A78" s="11" t="n"/>
-      <c r="B78" s="11" t="n"/>
-      <c r="C78" s="11" t="n"/>
-      <c r="D78" s="12" t="n"/>
-      <c r="E78" s="11" t="n"/>
-      <c r="F78" s="11" t="n"/>
-      <c r="G78" s="11" t="n"/>
-      <c r="H78" s="13" t="n"/>
-      <c r="I78" s="12" t="n"/>
-      <c r="J78" s="12" t="n"/>
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t>Confidential (family-owned technical installer)</t>
+        </is>
+      </c>
+      <c r="B78" s="17" t="inlineStr">
+        <is>
+          <t>Junior Project Leader Techniques</t>
+        </is>
+      </c>
+      <c r="C78" s="17" t="inlineStr">
+        <is>
+          <t>Poperinge, BE</t>
+        </is>
+      </c>
+      <c r="D78" s="18" t="n"/>
+      <c r="E78" s="17" t="n"/>
+      <c r="F78" s="17" t="inlineStr">
+        <is>
+          <t>Job Board</t>
+        </is>
+      </c>
+      <c r="G78" s="17" t="n"/>
+      <c r="H78" s="19" t="n">
+        <v>46255</v>
+      </c>
+      <c r="I78" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J78" s="18" t="n"/>
       <c r="K78" s="14">
         <f>IF($H78="","",TODAY()-$H78)</f>
         <v/>
       </c>
-      <c r="L78" s="13" t="n"/>
-      <c r="M78" s="11" t="n"/>
-      <c r="N78" s="13" t="n"/>
-      <c r="O78" s="11" t="n"/>
-      <c r="P78" s="11" t="n"/>
-      <c r="Q78" s="11" t="n"/>
-      <c r="R78" s="12" t="n"/>
-      <c r="S78" s="11" t="n"/>
+      <c r="L78" s="19" t="n"/>
+      <c r="M78" s="17" t="n"/>
+      <c r="N78" s="19" t="n"/>
+      <c r="O78" s="17" t="n"/>
+      <c r="P78" s="17" t="n"/>
+      <c r="Q78" s="17" t="inlineStr">
+        <is>
+          <t>belgium/2026_08_21_poperinge_junior_project_leader</t>
+        </is>
+      </c>
+      <c r="R78" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S78" s="17" t="inlineStr">
+        <is>
+          <t>Long-shot: client-facing HVAC/technical PM role in West Flanders, likely requires Dutch which the candidate does not have. Applied at user's request with cover letter transparent about English working language and commitment to learn Dutch.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="21">
       <c r="A79" s="11" t="n"/>

</xml_diff>

<commit_message>
Add Drees & Sommer Junior BIM Manager row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6445,28 +6445,66 @@
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="21">
-      <c r="A79" s="11" t="n"/>
-      <c r="B79" s="11" t="n"/>
-      <c r="C79" s="11" t="n"/>
-      <c r="D79" s="12" t="n"/>
-      <c r="E79" s="11" t="n"/>
-      <c r="F79" s="11" t="n"/>
-      <c r="G79" s="11" t="n"/>
-      <c r="H79" s="13" t="n"/>
-      <c r="I79" s="12" t="n"/>
-      <c r="J79" s="12" t="n"/>
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t>Drees &amp; Sommer</t>
+        </is>
+      </c>
+      <c r="B79" s="17" t="inlineStr">
+        <is>
+          <t>(Junior) BIM Manager (m/f/d)</t>
+        </is>
+      </c>
+      <c r="C79" s="17" t="inlineStr">
+        <is>
+          <t>Leipzig, DE</t>
+        </is>
+      </c>
+      <c r="D79" s="18" t="n"/>
+      <c r="E79" s="17" t="n"/>
+      <c r="F79" s="17" t="inlineStr">
+        <is>
+          <t>Company Site</t>
+        </is>
+      </c>
+      <c r="G79" s="17" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/DreesSommerSE/744000133970415--junior-bim-manager-w-m-d-</t>
+        </is>
+      </c>
+      <c r="H79" s="19" t="n">
+        <v>46259</v>
+      </c>
+      <c r="I79" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J79" s="18" t="n"/>
       <c r="K79" s="14">
         <f>IF($H79="","",TODAY()-$H79)</f>
         <v/>
       </c>
-      <c r="L79" s="13" t="n"/>
-      <c r="M79" s="11" t="n"/>
-      <c r="N79" s="13" t="n"/>
-      <c r="O79" s="11" t="n"/>
-      <c r="P79" s="11" t="n"/>
-      <c r="Q79" s="11" t="n"/>
-      <c r="R79" s="12" t="n"/>
-      <c r="S79" s="11" t="n"/>
+      <c r="L79" s="19" t="n"/>
+      <c r="M79" s="17" t="n"/>
+      <c r="N79" s="19" t="n"/>
+      <c r="O79" s="17" t="n"/>
+      <c r="P79" s="17" t="n"/>
+      <c r="Q79" s="17" t="inlineStr">
+        <is>
+          <t>germany/2026_08_25_drees_sommer_junior_bim_manager</t>
+        </is>
+      </c>
+      <c r="R79" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S79" s="17" t="inlineStr">
+        <is>
+          <t>Strong entry-level fit: BIM methodology implementation, cross-discipline coordination, and stakeholder-facing communication line up directly with the role. No photo included (standing gap, confirmed with user, no asset available).</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="21">
       <c r="A80" s="11" t="n"/>

</xml_diff>

<commit_message>
Add CYPE BIM software developer referral row to Job Application Tracker
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -6507,28 +6507,62 @@
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="21">
-      <c r="A80" s="11" t="n"/>
-      <c r="B80" s="11" t="n"/>
-      <c r="C80" s="11" t="n"/>
-      <c r="D80" s="12" t="n"/>
-      <c r="E80" s="11" t="n"/>
-      <c r="F80" s="11" t="n"/>
-      <c r="G80" s="11" t="n"/>
-      <c r="H80" s="13" t="n"/>
-      <c r="I80" s="12" t="n"/>
-      <c r="J80" s="12" t="n"/>
+      <c r="A80" s="17" t="inlineStr">
+        <is>
+          <t>CYPE</t>
+        </is>
+      </c>
+      <c r="B80" s="17" t="inlineStr">
+        <is>
+          <t>BIM Software Developer (R&amp;D / interoperability, referral)</t>
+        </is>
+      </c>
+      <c r="C80" s="17" t="inlineStr">
+        <is>
+          <t>Alicante, ES</t>
+        </is>
+      </c>
+      <c r="D80" s="18" t="n"/>
+      <c r="E80" s="17" t="n"/>
+      <c r="F80" s="17" t="inlineStr">
+        <is>
+          <t>Referral</t>
+        </is>
+      </c>
+      <c r="G80" s="17" t="n"/>
+      <c r="H80" s="19" t="n">
+        <v>46261</v>
+      </c>
+      <c r="I80" s="18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="J80" s="18" t="n"/>
       <c r="K80" s="14">
         <f>IF($H80="","",TODAY()-$H80)</f>
         <v/>
       </c>
-      <c r="L80" s="13" t="n"/>
-      <c r="M80" s="11" t="n"/>
-      <c r="N80" s="13" t="n"/>
-      <c r="O80" s="11" t="n"/>
-      <c r="P80" s="11" t="n"/>
-      <c r="Q80" s="11" t="n"/>
-      <c r="R80" s="12" t="n"/>
-      <c r="S80" s="11" t="n"/>
+      <c r="L80" s="19" t="n"/>
+      <c r="M80" s="17" t="n"/>
+      <c r="N80" s="19" t="n"/>
+      <c r="O80" s="17" t="n"/>
+      <c r="P80" s="17" t="n"/>
+      <c r="Q80" s="17" t="inlineStr">
+        <is>
+          <t>spain/2026_08_27_cype_bim_software_referral</t>
+        </is>
+      </c>
+      <c r="R80" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="S80" s="17" t="inlineStr">
+        <is>
+          <t>Warm personal referral from an outgoing employee (R&amp;D on Horizon/LIFE EU projects plus BIM software interoperability with Revit). CV tailored toward software side (IfcToNeo4j, BIMGraphExplorer, Headstarter AI fellowship, in-progress That Open Company BIM software dev programme). No formal job posting/link.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="21">
       <c r="A81" s="11" t="n"/>

</xml_diff>